<commit_message>
fix: agregar combos por persona de banquetes primavera con enlaces correspondientes
</commit_message>
<xml_diff>
--- a/assets/Smart_Event_Planner_Pro.xlsx
+++ b/assets/Smart_Event_Planner_Pro.xlsx
@@ -1671,7 +1671,7 @@
       <c r="H13" s="114" t="n"/>
       <c r="I13" s="114" t="n"/>
       <c r="J13" s="126">
-        <f>COUNTIF('📦 Catálogo'!G5:G116,"✓")</f>
+        <f>COUNTIF('📦 Catálogo'!G5:G118,"✓")</f>
         <v/>
       </c>
       <c r="K13" s="114" t="n"/>
@@ -3653,7 +3653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J117"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="106" min="1" max="1"/>
@@ -4201,16 +4201,16 @@
       </c>
       <c r="C18" s="218" t="inlineStr">
         <is>
-          <t>Banquetes Primavera - Gala 3 Tiempos</t>
+          <t>Banquetes Primavera - Combo Básico (Por Persona)</t>
         </is>
       </c>
       <c r="D18" s="218" t="inlineStr">
         <is>
-          <t>Entrada, plato fuerte y postre. Vajilla, cristalería y servicio de gala.</t>
+          <t>Mínimo 100 personas. Banquete 3 tiempos, torna fiesta, DJ profesional, montaje con flor natural y coordinador.</t>
         </is>
       </c>
       <c r="E18" s="219" t="n">
-        <v>40950</v>
+        <v>993</v>
       </c>
       <c r="F18" s="220" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="H18" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Combos Oficiales")</f>
         <v/>
       </c>
       <c r="I18" s="216" t="n"/>
@@ -4239,16 +4239,16 @@
       </c>
       <c r="C19" s="218" t="inlineStr">
         <is>
-          <t>Banquetes Primavera - Buffet Especial</t>
+          <t>Banquetes Primavera - Combo de Lujo (Por Persona)</t>
         </is>
       </c>
       <c r="D19" s="218" t="inlineStr">
         <is>
-          <t>Variedad de guisados de gala a libre servicio para tus invitados.</t>
+          <t>Mínimo 100 personas. Incluye salón techado, cóctel de bienvenida, banquete, torna fiesta, DJ avanzado y montaje premium.</t>
         </is>
       </c>
       <c r="E19" s="219" t="n">
-        <v>32760</v>
+        <v>1169</v>
       </c>
       <c r="F19" s="220" t="inlineStr">
         <is>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="H19" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Combos Oficiales")</f>
         <v/>
       </c>
       <c r="I19" s="216" t="n"/>
@@ -4277,20 +4277,20 @@
       </c>
       <c r="C20" s="218" t="inlineStr">
         <is>
-          <t>Banquetes Primavera - Tornaboda Chilaquiles</t>
+          <t>Banquetes Primavera - Gala 3 Tiempos</t>
         </is>
       </c>
       <c r="D20" s="218" t="inlineStr">
         <is>
-          <t>Chilaquiles rojos/verdes al cierre del evento (100 personas).</t>
+          <t>Entrada, plato fuerte y postre. Vajilla, cristalería y servicio de gala.</t>
         </is>
       </c>
       <c r="E20" s="219" t="n">
-        <v>7020</v>
+        <v>40950</v>
       </c>
       <c r="F20" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G20" s="217" t="inlineStr">
@@ -4315,20 +4315,20 @@
       </c>
       <c r="C21" s="218" t="inlineStr">
         <is>
-          <t>Mesa de postres</t>
+          <t>Banquetes Primavera - Buffet Especial</t>
         </is>
       </c>
       <c r="D21" s="218" t="inlineStr">
         <is>
-          <t>Variedad de dulces y postres artesanales montados sobre mesa temática.</t>
+          <t>Variedad de guisados de gala a libre servicio para tus invitados.</t>
         </is>
       </c>
       <c r="E21" s="219" t="n">
-        <v>4500</v>
+        <v>32760</v>
       </c>
       <c r="F21" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G21" s="217" t="inlineStr">
@@ -4336,7 +4336,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H21" s="218" t="inlineStr"/>
+      <c r="H21" s="218">
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <v/>
+      </c>
       <c r="I21" s="216" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1" s="107">
@@ -4350,20 +4353,20 @@
       </c>
       <c r="C22" s="218" t="inlineStr">
         <is>
-          <t>Pastel de bodas/XV</t>
+          <t>Banquetes Primavera - Tornaboda Chilaquiles</t>
         </is>
       </c>
       <c r="D22" s="218" t="inlineStr">
         <is>
-          <t>Pastel artístico o tradicional diseñado a medida.</t>
+          <t>Chilaquiles rojos/verdes al cierre del evento (100 personas).</t>
         </is>
       </c>
       <c r="E22" s="219" t="n">
-        <v>8000</v>
+        <v>7020</v>
       </c>
       <c r="F22" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G22" s="217" t="inlineStr">
@@ -4371,7 +4374,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H22" s="218" t="inlineStr"/>
+      <c r="H22" s="218">
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <v/>
+      </c>
       <c r="I22" s="216" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1" s="107">
@@ -4385,16 +4391,16 @@
       </c>
       <c r="C23" s="218" t="inlineStr">
         <is>
-          <t>Candy bar</t>
+          <t>Mesa de postres</t>
         </is>
       </c>
       <c r="D23" s="218" t="inlineStr">
         <is>
-          <t>Barra de golosinas y dulces decorativa.</t>
+          <t>Variedad de dulces y postres artesanales montados sobre mesa temática.</t>
         </is>
       </c>
       <c r="E23" s="219" t="n">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="F23" s="220" t="inlineStr">
         <is>
@@ -4420,16 +4426,16 @@
       </c>
       <c r="C24" s="218" t="inlineStr">
         <is>
-          <t>Barra libre</t>
+          <t>Pastel de bodas/XV</t>
         </is>
       </c>
       <c r="D24" s="218" t="inlineStr">
         <is>
-          <t>Bebidas nacionales ilimitadas durante 5 horas.</t>
+          <t>Pastel artístico o tradicional diseñado a medida.</t>
         </is>
       </c>
       <c r="E24" s="219" t="n">
-        <v>12000</v>
+        <v>8000</v>
       </c>
       <c r="F24" s="220" t="inlineStr">
         <is>
@@ -4455,16 +4461,16 @@
       </c>
       <c r="C25" s="218" t="inlineStr">
         <is>
-          <t>Mixología Primavera</t>
+          <t>Candy bar</t>
         </is>
       </c>
       <c r="D25" s="218" t="inlineStr">
         <is>
-          <t>Cócteles artesanales y presentaciones con alcohol y sin alcohol.</t>
+          <t>Barra de golosinas y dulces de diseño.</t>
         </is>
       </c>
       <c r="E25" s="219" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="F25" s="220" t="inlineStr">
         <is>
@@ -4490,20 +4496,20 @@
       </c>
       <c r="C26" s="218" t="inlineStr">
         <is>
-          <t>Paleteria La Princesa - Paquete 1</t>
+          <t>Barra libre</t>
         </is>
       </c>
       <c r="D26" s="218" t="inlineStr">
         <is>
-          <t>Carrito personalizado con 150 mini paletas tradicionales de fruta natural.</t>
+          <t>Bebidas nacionales ilimitadas durante 5 horas.</t>
         </is>
       </c>
       <c r="E26" s="219" t="n">
-        <v>1989</v>
+        <v>12000</v>
       </c>
       <c r="F26" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G26" s="217" t="inlineStr">
@@ -4511,10 +4517,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H26" s="218">
-        <f>HYPERLINK("https://wa.me/527772141981","Pedir La Princesa")</f>
-        <v/>
-      </c>
+      <c r="H26" s="218" t="inlineStr"/>
       <c r="I26" s="216" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="107">
@@ -4528,16 +4531,16 @@
       </c>
       <c r="C27" s="218" t="inlineStr">
         <is>
-          <t>Paleteria La Princesa - Paquete 2</t>
+          <t>Mixología Primavera</t>
         </is>
       </c>
       <c r="D27" s="218" t="inlineStr">
         <is>
-          <t>Servicio de Nieve y Helado artesanal de Michoacán para 100 personas.</t>
+          <t>Cócteles artesanales y presentaciones con alcohol y sin alcohol.</t>
         </is>
       </c>
       <c r="E27" s="219" t="n">
-        <v>4212</v>
+        <v>5000</v>
       </c>
       <c r="F27" s="220" t="inlineStr">
         <is>
@@ -4549,10 +4552,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H27" s="218">
-        <f>HYPERLINK("https://wa.me/527772141981","Pedir La Princesa")</f>
-        <v/>
-      </c>
+      <c r="H27" s="218" t="inlineStr"/>
       <c r="I27" s="216" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1" s="107">
@@ -4566,16 +4566,16 @@
       </c>
       <c r="C28" s="218" t="inlineStr">
         <is>
-          <t>Paleteria La Princesa - Paquete 3</t>
+          <t>Paleteria La Princesa - Paquete 1</t>
         </is>
       </c>
       <c r="D28" s="218" t="inlineStr">
         <is>
-          <t>Servicio Mixto: 75 mini paletas + Helado/Nieve para 50 personas.</t>
+          <t>Carrito personalizado con 150 mini paletas tradicionales de fruta natural.</t>
         </is>
       </c>
       <c r="E28" s="219" t="n">
-        <v>3042</v>
+        <v>1989</v>
       </c>
       <c r="F28" s="220" t="inlineStr">
         <is>
@@ -4604,20 +4604,20 @@
       </c>
       <c r="C29" s="218" t="inlineStr">
         <is>
-          <t>Tequila Don Ramón - Luis Miguel Plata</t>
+          <t>Paleteria La Princesa - Paquete 2</t>
         </is>
       </c>
       <c r="D29" s="218" t="inlineStr">
         <is>
-          <t>Botella Cerámica Personalizada con grabado punta diamante (Plata).</t>
+          <t>Servicio de Nieve y Helado artesanal de Michoacán para 100 personas.</t>
         </is>
       </c>
       <c r="E29" s="219" t="n">
-        <v>6435</v>
+        <v>4212</v>
       </c>
       <c r="F29" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G29" s="217" t="inlineStr">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="H29" s="218">
-        <f>HYPERLINK("https://wa.me/527771204557","Pedir Don Ramon")</f>
+        <f>HYPERLINK("https://wa.me/527772141981","Pedir La Princesa")</f>
         <v/>
       </c>
       <c r="I29" s="216" t="n"/>
@@ -4642,20 +4642,20 @@
       </c>
       <c r="C30" s="218" t="inlineStr">
         <is>
-          <t>Tequila Don Ramón - Luis Miguel Reposado</t>
+          <t>Paleteria La Princesa - Paquete 3</t>
         </is>
       </c>
       <c r="D30" s="218" t="inlineStr">
         <is>
-          <t>Botella Cerámica Personalizada con grabado punta diamante (Reposado).</t>
+          <t>Servicio Mixto: 75 mini paletas + Helado/Nieve para 50 personas.</t>
         </is>
       </c>
       <c r="E30" s="219" t="n">
-        <v>7465</v>
+        <v>3042</v>
       </c>
       <c r="F30" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G30" s="217" t="inlineStr">
@@ -4664,7 +4664,7 @@
         </is>
       </c>
       <c r="H30" s="218">
-        <f>HYPERLINK("https://wa.me/527771204557","Pedir Don Ramon")</f>
+        <f>HYPERLINK("https://wa.me/527772141981","Pedir La Princesa")</f>
         <v/>
       </c>
       <c r="I30" s="216" t="n"/>
@@ -4680,16 +4680,16 @@
       </c>
       <c r="C31" s="218" t="inlineStr">
         <is>
-          <t>Tequila Don Ramón - Luis Miguel Añejo</t>
+          <t>Tequila Don Ramón - Luis Miguel Plata</t>
         </is>
       </c>
       <c r="D31" s="218" t="inlineStr">
         <is>
-          <t>Botella Cerámica Personalizada con grabado punta diamante (Añejo).</t>
+          <t>Botella Cerámica Personalizada con grabado punta diamante (Plata).</t>
         </is>
       </c>
       <c r="E31" s="219" t="n">
-        <v>8752</v>
+        <v>6435</v>
       </c>
       <c r="F31" s="220" t="inlineStr">
         <is>
@@ -4718,16 +4718,16 @@
       </c>
       <c r="C32" s="218" t="inlineStr">
         <is>
-          <t>Tequila Don Ramón - Swarovski Plata</t>
+          <t>Tequila Don Ramón - Luis Miguel Reposado</t>
         </is>
       </c>
       <c r="D32" s="218" t="inlineStr">
         <is>
-          <t>Edición Coleccionista con cristales incrustados (Plata).</t>
+          <t>Botella Cerámica Personalizada con grabado punta diamante (Reposado).</t>
         </is>
       </c>
       <c r="E32" s="219" t="n">
-        <v>9565</v>
+        <v>7465</v>
       </c>
       <c r="F32" s="220" t="inlineStr">
         <is>
@@ -4756,16 +4756,16 @@
       </c>
       <c r="C33" s="218" t="inlineStr">
         <is>
-          <t>Tequila Don Ramón - Swarovski Añejo</t>
+          <t>Tequila Don Ramón - Luis Miguel Añejo</t>
         </is>
       </c>
       <c r="D33" s="218" t="inlineStr">
         <is>
-          <t>Edición Coleccionista con cristales incrustados (Añejo).</t>
+          <t>Botella Cerámica Personalizada con grabado punta diamante (Añejo).</t>
         </is>
       </c>
       <c r="E33" s="219" t="n">
-        <v>10723</v>
+        <v>8752</v>
       </c>
       <c r="F33" s="220" t="inlineStr">
         <is>
@@ -4794,16 +4794,16 @@
       </c>
       <c r="C34" s="218" t="inlineStr">
         <is>
-          <t>Tequila Don Ramón - Swarovski Extra Añejo</t>
+          <t>Tequila Don Ramón - Swarovski Plata</t>
         </is>
       </c>
       <c r="D34" s="218" t="inlineStr">
         <is>
-          <t>Edición Coleccionista con cristales incrustados (Extra Añejo).</t>
+          <t>Edición Coleccionista con cristales incrustados (Plata).</t>
         </is>
       </c>
       <c r="E34" s="219" t="n">
-        <v>12525</v>
+        <v>9565</v>
       </c>
       <c r="F34" s="220" t="inlineStr">
         <is>
@@ -4822,41 +4822,64 @@
       <c r="I34" s="216" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1" s="107">
-      <c r="A35" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Entretenimiento</t>
-        </is>
-      </c>
-      <c r="B35" s="216" t="n"/>
-      <c r="C35" s="216" t="n"/>
-      <c r="D35" s="216" t="n"/>
-      <c r="E35" s="216" t="n"/>
-      <c r="F35" s="216" t="n"/>
-      <c r="G35" s="216" t="n"/>
-      <c r="H35" s="216" t="n"/>
+      <c r="A35" s="217" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="218" t="inlineStr">
+        <is>
+          <t>Banquete &amp; Bebidas</t>
+        </is>
+      </c>
+      <c r="C35" s="218" t="inlineStr">
+        <is>
+          <t>Tequila Don Ramón - Swarovski Añejo</t>
+        </is>
+      </c>
+      <c r="D35" s="218" t="inlineStr">
+        <is>
+          <t>Edición Coleccionista con cristales incrustados (Añejo).</t>
+        </is>
+      </c>
+      <c r="E35" s="219" t="n">
+        <v>10723</v>
+      </c>
+      <c r="F35" s="220" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G35" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="218">
+        <f>HYPERLINK("https://wa.me/527771204557","Pedir Don Ramon")</f>
+        <v/>
+      </c>
       <c r="I35" s="216" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1" s="107">
       <c r="A36" s="217" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B36" s="218" t="inlineStr">
         <is>
-          <t>Entretenimiento</t>
+          <t>Banquete &amp; Bebidas</t>
         </is>
       </c>
       <c r="C36" s="218" t="inlineStr">
         <is>
-          <t>Scanner DJ - Paquete Básico</t>
+          <t>Tequila Don Ramón - Swarovski Extra Añejo</t>
         </is>
       </c>
       <c r="D36" s="218" t="inlineStr">
         <is>
-          <t>DJ profesional, audio estándar e iluminación LED.</t>
+          <t>Edición Coleccionista con cristales incrustados (Extra Añejo).</t>
         </is>
       </c>
       <c r="E36" s="219" t="n">
-        <v>11700</v>
+        <v>12525</v>
       </c>
       <c r="F36" s="220" t="inlineStr">
         <is>
@@ -4869,47 +4892,24 @@
         </is>
       </c>
       <c r="H36" s="218">
-        <f>HYPERLINK("https://wa.me/527771992434","Pedir Scanner DJ")</f>
+        <f>HYPERLINK("https://wa.me/527771204557","Pedir Don Ramon")</f>
         <v/>
       </c>
       <c r="I36" s="216" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1" s="107">
-      <c r="A37" s="217" t="n">
-        <v>31</v>
-      </c>
-      <c r="B37" s="218" t="inlineStr">
-        <is>
-          <t>Entretenimiento</t>
-        </is>
-      </c>
-      <c r="C37" s="218" t="inlineStr">
-        <is>
-          <t>Scanner DJ - Paquete Intermedio</t>
-        </is>
-      </c>
-      <c r="D37" s="218" t="inlineStr">
-        <is>
-          <t>Audio premium, cabina de DJ iluminada y luces robóticas.</t>
-        </is>
-      </c>
-      <c r="E37" s="219" t="n">
-        <v>17550</v>
-      </c>
-      <c r="F37" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G37" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="218">
-        <f>HYPERLINK("https://wa.me/527771992434","Pedir Scanner DJ")</f>
-        <v/>
-      </c>
+      <c r="A37" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Entretenimiento</t>
+        </is>
+      </c>
+      <c r="B37" s="216" t="n"/>
+      <c r="C37" s="216" t="n"/>
+      <c r="D37" s="216" t="n"/>
+      <c r="E37" s="216" t="n"/>
+      <c r="F37" s="216" t="n"/>
+      <c r="G37" s="216" t="n"/>
+      <c r="H37" s="216" t="n"/>
       <c r="I37" s="216" t="n"/>
     </row>
     <row r="38" ht="19.5" customHeight="1" s="107">
@@ -4923,16 +4923,16 @@
       </c>
       <c r="C38" s="218" t="inlineStr">
         <is>
-          <t>Scanner DJ - Paquete Completo</t>
+          <t>Scanner DJ - Paquete Básico</t>
         </is>
       </c>
       <c r="D38" s="218" t="inlineStr">
         <is>
-          <t>Mega producción de audio, pantallas y show de luces robotizadas.</t>
+          <t>DJ profesional, audio estándar e iluminación LED.</t>
         </is>
       </c>
       <c r="E38" s="219" t="n">
-        <v>23400</v>
+        <v>11700</v>
       </c>
       <c r="F38" s="220" t="inlineStr">
         <is>
@@ -4961,16 +4961,16 @@
       </c>
       <c r="C39" s="218" t="inlineStr">
         <is>
-          <t>Corona Music - Paquete Mediano</t>
+          <t>Scanner DJ - Paquete Intermedio</t>
         </is>
       </c>
       <c r="D39" s="218" t="inlineStr">
         <is>
-          <t>DJ, Iluminación profesional y audio de alta fidelidad.</t>
+          <t>Audio premium, cabina de DJ iluminada y luces robóticas.</t>
         </is>
       </c>
       <c r="E39" s="219" t="n">
-        <v>10530</v>
+        <v>17550</v>
       </c>
       <c r="F39" s="220" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
         </is>
       </c>
       <c r="H39" s="218">
-        <f>HYPERLINK("https://wa.me/527774458481","Pedir Corona Music")</f>
+        <f>HYPERLINK("https://wa.me/527771992434","Pedir Scanner DJ")</f>
         <v/>
       </c>
       <c r="I39" s="216" t="n"/>
@@ -4999,16 +4999,16 @@
       </c>
       <c r="C40" s="218" t="inlineStr">
         <is>
-          <t>Corona Music - Paquete VIP</t>
+          <t>Scanner DJ - Paquete Completo</t>
         </is>
       </c>
       <c r="D40" s="218" t="inlineStr">
         <is>
-          <t>Producción de audio premium, pantallas LED, cabina y pista iluminada.</t>
+          <t>Mega producción de audio, pantallas y show de luces robotizadas.</t>
         </is>
       </c>
       <c r="E40" s="219" t="n">
-        <v>18720</v>
+        <v>23400</v>
       </c>
       <c r="F40" s="220" t="inlineStr">
         <is>
@@ -5021,7 +5021,7 @@
         </is>
       </c>
       <c r="H40" s="218">
-        <f>HYPERLINK("https://wa.me/527774458481","Pedir Corona Music")</f>
+        <f>HYPERLINK("https://wa.me/527771992434","Pedir Scanner DJ")</f>
         <v/>
       </c>
       <c r="I40" s="216" t="n"/>
@@ -5037,20 +5037,20 @@
       </c>
       <c r="C41" s="218" t="inlineStr">
         <is>
-          <t>Mariachi Xiuhtepetl - Dos Horas</t>
+          <t>Corona Music - Paquete Mediano</t>
         </is>
       </c>
       <c r="D41" s="218" t="inlineStr">
         <is>
-          <t>Show de Mariachi tradicional completo con arpa en vivo (2 horas).</t>
+          <t>DJ, Iluminación profesional y audio de alta fidelidad.</t>
         </is>
       </c>
       <c r="E41" s="219" t="n">
-        <v>11115</v>
+        <v>10530</v>
       </c>
       <c r="F41" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G41" s="217" t="inlineStr">
@@ -5059,7 +5059,7 @@
         </is>
       </c>
       <c r="H41" s="218">
-        <f>HYPERLINK("https://wa.me/527771204557","Pedir Mariachi")</f>
+        <f>HYPERLINK("https://wa.me/527774458481","Pedir Corona Music")</f>
         <v/>
       </c>
       <c r="I41" s="216" t="n"/>
@@ -5075,20 +5075,20 @@
       </c>
       <c r="C42" s="218" t="inlineStr">
         <is>
-          <t>Mariachi Xiuhtepetl - Una Hora</t>
+          <t>Corona Music - Paquete VIP</t>
         </is>
       </c>
       <c r="D42" s="218" t="inlineStr">
         <is>
-          <t>Show de Mariachi tradicional completo con arpa en vivo (1 hora).</t>
+          <t>Producción de audio premium, pantallas LED, cabina y pista iluminada.</t>
         </is>
       </c>
       <c r="E42" s="219" t="n">
-        <v>5850</v>
+        <v>18720</v>
       </c>
       <c r="F42" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G42" s="217" t="inlineStr">
@@ -5097,7 +5097,7 @@
         </is>
       </c>
       <c r="H42" s="218">
-        <f>HYPERLINK("https://wa.me/527771204557","Pedir Mariachi")</f>
+        <f>HYPERLINK("https://wa.me/527774458481","Pedir Corona Music")</f>
         <v/>
       </c>
       <c r="I42" s="216" t="n"/>
@@ -5113,16 +5113,16 @@
       </c>
       <c r="C43" s="218" t="inlineStr">
         <is>
-          <t>Mariachi Xiuhtepetl - Set 45 Min</t>
+          <t>Mariachi Xiuhtepetl - Dos Horas</t>
         </is>
       </c>
       <c r="D43" s="218" t="inlineStr">
         <is>
-          <t>Set rápido de 45 minutos ideal para cenas o recepciones.</t>
+          <t>Show de Mariachi tradicional completo con arpa en vivo (2 horas).</t>
         </is>
       </c>
       <c r="E43" s="219" t="n">
-        <v>5265</v>
+        <v>11115</v>
       </c>
       <c r="F43" s="220" t="inlineStr">
         <is>
@@ -5151,16 +5151,16 @@
       </c>
       <c r="C44" s="218" t="inlineStr">
         <is>
-          <t>Mariachi Xiuhtepetl - Serenata</t>
+          <t>Mariachi Xiuhtepetl - Una Hora</t>
         </is>
       </c>
       <c r="D44" s="218" t="inlineStr">
         <is>
-          <t>Serenata tradicional completa de 10 canciones.</t>
+          <t>Show de Mariachi tradicional completo con arpa en vivo (1 hora).</t>
         </is>
       </c>
       <c r="E44" s="219" t="n">
-        <v>4680</v>
+        <v>5850</v>
       </c>
       <c r="F44" s="220" t="inlineStr">
         <is>
@@ -5189,16 +5189,16 @@
       </c>
       <c r="C45" s="218" t="inlineStr">
         <is>
-          <t>Mariachi Xiuhtepetl - Serenata Corta</t>
+          <t>Mariachi Xiuhtepetl - Set 45 Min</t>
         </is>
       </c>
       <c r="D45" s="218" t="inlineStr">
         <is>
-          <t>Serenata corta de 5 canciones.</t>
+          <t>Set rápido de 45 minutos ideal para cenas o recepciones.</t>
         </is>
       </c>
       <c r="E45" s="219" t="n">
-        <v>4095</v>
+        <v>5265</v>
       </c>
       <c r="F45" s="220" t="inlineStr">
         <is>
@@ -5227,16 +5227,16 @@
       </c>
       <c r="C46" s="218" t="inlineStr">
         <is>
-          <t>Saxofonista</t>
+          <t>Mariachi Xiuhtepetl - Serenata</t>
         </is>
       </c>
       <c r="D46" s="218" t="inlineStr">
         <is>
-          <t>Música de saxofón en vivo para el banquete o cocktail.</t>
+          <t>Serenata tradicional completa de 10 canciones.</t>
         </is>
       </c>
       <c r="E46" s="219" t="n">
-        <v>3500</v>
+        <v>4680</v>
       </c>
       <c r="F46" s="220" t="inlineStr">
         <is>
@@ -5248,7 +5248,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H46" s="218" t="inlineStr"/>
+      <c r="H46" s="218">
+        <f>HYPERLINK("https://wa.me/527771204557","Pedir Mariachi")</f>
+        <v/>
+      </c>
       <c r="I46" s="216" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="107">
@@ -5262,16 +5265,16 @@
       </c>
       <c r="C47" s="218" t="inlineStr">
         <is>
-          <t>Violinista</t>
+          <t>Mariachi Xiuhtepetl - Serenata Corta</t>
         </is>
       </c>
       <c r="D47" s="218" t="inlineStr">
         <is>
-          <t>Música instrumental de violín para ceremonia o cena.</t>
+          <t>Serenata corta de 5 canciones.</t>
         </is>
       </c>
       <c r="E47" s="219" t="n">
-        <v>3000</v>
+        <v>4095</v>
       </c>
       <c r="F47" s="220" t="inlineStr">
         <is>
@@ -5283,7 +5286,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H47" s="218" t="inlineStr"/>
+      <c r="H47" s="218">
+        <f>HYPERLINK("https://wa.me/527771204557","Pedir Mariachi")</f>
+        <v/>
+      </c>
       <c r="I47" s="216" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1" s="107">
@@ -5297,16 +5303,16 @@
       </c>
       <c r="C48" s="218" t="inlineStr">
         <is>
-          <t>Batucada</t>
+          <t>Saxofonista</t>
         </is>
       </c>
       <c r="D48" s="218" t="inlineStr">
         <is>
-          <t>Show interactivo de percusión con globos y antifaces.</t>
+          <t>Música de saxofón en vivo para el banquete o cocktail.</t>
         </is>
       </c>
       <c r="E48" s="219" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="F48" s="220" t="inlineStr">
         <is>
@@ -5332,16 +5338,16 @@
       </c>
       <c r="C49" s="218" t="inlineStr">
         <is>
-          <t>Cabina de fotos / Photo booth</t>
+          <t>Violinista</t>
         </is>
       </c>
       <c r="D49" s="218" t="inlineStr">
         <is>
-          <t>Fotos instantáneas con accesorios de diversión.</t>
+          <t>Música instrumental de violín para ceremonia o cena.</t>
         </is>
       </c>
       <c r="E49" s="219" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="F49" s="220" t="inlineStr">
         <is>
@@ -5357,45 +5363,65 @@
       <c r="I49" s="216" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="107">
-      <c r="A50" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Foto &amp; Video</t>
-        </is>
-      </c>
-      <c r="B50" s="216" t="n"/>
-      <c r="C50" s="216" t="n"/>
-      <c r="D50" s="216" t="n"/>
-      <c r="E50" s="216" t="n"/>
-      <c r="F50" s="216" t="n"/>
-      <c r="G50" s="216" t="n"/>
-      <c r="H50" s="216" t="n"/>
+      <c r="A50" s="217" t="n">
+        <v>44</v>
+      </c>
+      <c r="B50" s="218" t="inlineStr">
+        <is>
+          <t>Entretenimiento</t>
+        </is>
+      </c>
+      <c r="C50" s="218" t="inlineStr">
+        <is>
+          <t>Batucada</t>
+        </is>
+      </c>
+      <c r="D50" s="218" t="inlineStr">
+        <is>
+          <t>Show interactivo de percusión con globos y antifaces.</t>
+        </is>
+      </c>
+      <c r="E50" s="219" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F50" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G50" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="218" t="inlineStr"/>
       <c r="I50" s="216" t="n"/>
     </row>
     <row r="51" ht="19.5" customHeight="1" s="107">
       <c r="A51" s="217" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B51" s="218" t="inlineStr">
         <is>
-          <t>Foto &amp; Video</t>
+          <t>Entretenimiento</t>
         </is>
       </c>
       <c r="C51" s="218" t="inlineStr">
         <is>
-          <t>Licky Baut Photo - Cobertura Básica</t>
+          <t>Cabina de fotos / Photo booth</t>
         </is>
       </c>
       <c r="D51" s="218" t="inlineStr">
         <is>
-          <t>Cobertura de fotografía digital para ceremonia y banquete (5 horas).</t>
+          <t>Fotos instantáneas con accesorios de diversión.</t>
         </is>
       </c>
       <c r="E51" s="219" t="n">
-        <v>9360</v>
+        <v>4500</v>
       </c>
       <c r="F51" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G51" s="217" t="inlineStr">
@@ -5403,48 +5429,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H51" s="218">
-        <f>HYPERLINK("https://wa.me/527772967139","Pedir Licky Baut")</f>
-        <v/>
-      </c>
+      <c r="H51" s="218" t="inlineStr"/>
       <c r="I51" s="216" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1" s="107">
-      <c r="A52" s="217" t="n">
-        <v>45</v>
-      </c>
-      <c r="B52" s="218" t="inlineStr">
-        <is>
-          <t>Foto &amp; Video</t>
-        </is>
-      </c>
-      <c r="C52" s="218" t="inlineStr">
-        <is>
-          <t>Licky Baut Photo - Cinema VIP</t>
-        </is>
-      </c>
-      <c r="D52" s="218" t="inlineStr">
-        <is>
-          <t>Fotografía profesional + video cinematográfico editado + drone (toda la gala).</t>
-        </is>
-      </c>
-      <c r="E52" s="219" t="n">
-        <v>21060</v>
-      </c>
-      <c r="F52" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G52" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H52" s="218">
-        <f>HYPERLINK("https://wa.me/527772967139","Pedir Licky Baut")</f>
-        <v/>
-      </c>
+      <c r="A52" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Foto &amp; Video</t>
+        </is>
+      </c>
+      <c r="B52" s="216" t="n"/>
+      <c r="C52" s="216" t="n"/>
+      <c r="D52" s="216" t="n"/>
+      <c r="E52" s="216" t="n"/>
+      <c r="F52" s="216" t="n"/>
+      <c r="G52" s="216" t="n"/>
+      <c r="H52" s="216" t="n"/>
       <c r="I52" s="216" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1" s="107">
@@ -5458,20 +5458,20 @@
       </c>
       <c r="C53" s="218" t="inlineStr">
         <is>
-          <t>Drone</t>
+          <t>Licky Baut Photo - Cobertura Básica</t>
         </is>
       </c>
       <c r="D53" s="218" t="inlineStr">
         <is>
-          <t>Tomas aéreas de video en alta definición de la locación y el evento.</t>
+          <t>Cobertura de fotografía digital para ceremonia y banquete (5 horas).</t>
         </is>
       </c>
       <c r="E53" s="219" t="n">
-        <v>4000</v>
+        <v>9360</v>
       </c>
       <c r="F53" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G53" s="217" t="inlineStr">
@@ -5479,7 +5479,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H53" s="218" t="inlineStr"/>
+      <c r="H53" s="218">
+        <f>HYPERLINK("https://wa.me/527772967139","Pedir Licky Baut")</f>
+        <v/>
+      </c>
       <c r="I53" s="216" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1" s="107">
@@ -5493,20 +5496,20 @@
       </c>
       <c r="C54" s="218" t="inlineStr">
         <is>
-          <t>Same Day Edit</t>
+          <t>Licky Baut Photo - Cinema VIP</t>
         </is>
       </c>
       <c r="D54" s="218" t="inlineStr">
         <is>
-          <t>Video resumen proyectado antes de finalizar el evento.</t>
+          <t>Fotografía profesional + video cinematográfico editado + drone (toda la gala).</t>
         </is>
       </c>
       <c r="E54" s="219" t="n">
-        <v>3000</v>
+        <v>21060</v>
       </c>
       <c r="F54" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G54" s="217" t="inlineStr">
@@ -5514,7 +5517,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H54" s="218" t="inlineStr"/>
+      <c r="H54" s="218">
+        <f>HYPERLINK("https://wa.me/527772967139","Pedir Licky Baut")</f>
+        <v/>
+      </c>
       <c r="I54" s="216" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1" s="107">
@@ -5528,16 +5534,16 @@
       </c>
       <c r="C55" s="218" t="inlineStr">
         <is>
-          <t>Sesión pre-evento</t>
+          <t>Drone</t>
         </is>
       </c>
       <c r="D55" s="218" t="inlineStr">
         <is>
-          <t>Sesión fotográfica artística previa para novios o quinceañera.</t>
+          <t>Tomas aéreas de video en alta definición de la locación y el evento.</t>
         </is>
       </c>
       <c r="E55" s="219" t="n">
-        <v>3500</v>
+        <v>4000</v>
       </c>
       <c r="F55" s="220" t="inlineStr">
         <is>
@@ -5563,16 +5569,16 @@
       </c>
       <c r="C56" s="218" t="inlineStr">
         <is>
-          <t>Álbum impreso</t>
+          <t>Same Day Edit</t>
         </is>
       </c>
       <c r="D56" s="218" t="inlineStr">
         <is>
-          <t>Álbum fotográfico profesional de pasta dura personalizado.</t>
+          <t>Video resumen proyectado antes de finalizar el evento.</t>
         </is>
       </c>
       <c r="E56" s="219" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="F56" s="220" t="inlineStr">
         <is>
@@ -5588,45 +5594,65 @@
       <c r="I56" s="216" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1" s="107">
-      <c r="A57" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Belleza &amp; Imagen</t>
-        </is>
-      </c>
-      <c r="B57" s="216" t="n"/>
-      <c r="C57" s="216" t="n"/>
-      <c r="D57" s="216" t="n"/>
-      <c r="E57" s="216" t="n"/>
-      <c r="F57" s="216" t="n"/>
-      <c r="G57" s="216" t="n"/>
-      <c r="H57" s="216" t="n"/>
+      <c r="A57" s="217" t="n">
+        <v>50</v>
+      </c>
+      <c r="B57" s="218" t="inlineStr">
+        <is>
+          <t>Foto &amp; Video</t>
+        </is>
+      </c>
+      <c r="C57" s="218" t="inlineStr">
+        <is>
+          <t>Sesión pre-evento</t>
+        </is>
+      </c>
+      <c r="D57" s="218" t="inlineStr">
+        <is>
+          <t>Sesión fotográfica artística previa para novios o quinceañera.</t>
+        </is>
+      </c>
+      <c r="E57" s="219" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F57" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G57" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H57" s="218" t="inlineStr"/>
       <c r="I57" s="216" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1" s="107">
       <c r="A58" s="217" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B58" s="218" t="inlineStr">
         <is>
-          <t>Belleza &amp; Imagen</t>
+          <t>Foto &amp; Video</t>
         </is>
       </c>
       <c r="C58" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Paquete Plus Novia</t>
+          <t>Álbum impreso</t>
         </is>
       </c>
       <c r="D58" s="218" t="inlineStr">
         <is>
-          <t>Maquillaje aerógrafo en rostro, peinado, ampolleta de lifting e hidratación.</t>
+          <t>Álbum fotográfico profesional de pasta dura personalizado.</t>
         </is>
       </c>
       <c r="E58" s="219" t="n">
-        <v>10413</v>
+        <v>4500</v>
       </c>
       <c r="F58" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G58" s="217" t="inlineStr">
@@ -5634,48 +5660,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H58" s="218">
-        <f>HYPERLINK("https://wa.me/527774587923","Pedir Andrea Lozano")</f>
-        <v/>
-      </c>
+      <c r="H58" s="218" t="inlineStr"/>
       <c r="I58" s="216" t="n"/>
     </row>
     <row r="59" ht="19.5" customHeight="1" s="107">
-      <c r="A59" s="217" t="n">
-        <v>51</v>
-      </c>
-      <c r="B59" s="218" t="inlineStr">
-        <is>
-          <t>Belleza &amp; Imagen</t>
-        </is>
-      </c>
-      <c r="C59" s="218" t="inlineStr">
-        <is>
-          <t>Andrea Lozano - Paquete Power Novia</t>
-        </is>
-      </c>
-      <c r="D59" s="218" t="inlineStr">
-        <is>
-          <t>Maquillaje aerógrafo profesional y peinado de gala con tocado.</t>
-        </is>
-      </c>
-      <c r="E59" s="219" t="n">
-        <v>9009</v>
-      </c>
-      <c r="F59" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G59" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H59" s="218">
-        <f>HYPERLINK("https://wa.me/527774587923","Pedir Andrea Lozano")</f>
-        <v/>
-      </c>
+      <c r="A59" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Belleza &amp; Imagen</t>
+        </is>
+      </c>
+      <c r="B59" s="216" t="n"/>
+      <c r="C59" s="216" t="n"/>
+      <c r="D59" s="216" t="n"/>
+      <c r="E59" s="216" t="n"/>
+      <c r="F59" s="216" t="n"/>
+      <c r="G59" s="216" t="n"/>
+      <c r="H59" s="216" t="n"/>
       <c r="I59" s="216" t="n"/>
     </row>
     <row r="60" ht="18" customHeight="1" s="107">
@@ -5689,16 +5689,16 @@
       </c>
       <c r="C60" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Paquete Básico Novia</t>
+          <t>Andrea Lozano - Paquete Plus Novia</t>
         </is>
       </c>
       <c r="D60" s="218" t="inlineStr">
         <is>
-          <t>Maquillaje tradicional con pestañas y peinado profesional.</t>
+          <t>Maquillaje aerógrafo en rostro, peinado, ampolleta de lifting e hidratación.</t>
         </is>
       </c>
       <c r="E60" s="219" t="n">
-        <v>8424</v>
+        <v>10413</v>
       </c>
       <c r="F60" s="220" t="inlineStr">
         <is>
@@ -5727,20 +5727,20 @@
       </c>
       <c r="C61" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Maquillaje Aerógrafo Novia Ind</t>
+          <t>Andrea Lozano - Paquete Power Novia</t>
         </is>
       </c>
       <c r="D61" s="218" t="inlineStr">
         <is>
-          <t>Maquillaje aerógrafo individual para novia/quinceañera.</t>
+          <t>Maquillaje aerógrafo profesional y peinado de gala con tocado.</t>
         </is>
       </c>
       <c r="E61" s="219" t="n">
-        <v>2960</v>
+        <v>9009</v>
       </c>
       <c r="F61" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G61" s="217" t="inlineStr">
@@ -5765,20 +5765,20 @@
       </c>
       <c r="C62" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Maquillaje Tradicional Novia Ind</t>
+          <t>Andrea Lozano - Paquete Básico Novia</t>
         </is>
       </c>
       <c r="D62" s="218" t="inlineStr">
         <is>
-          <t>Maquillaje tradicional individual para novia/quinceañera.</t>
+          <t>Maquillaje tradicional con pestañas y peinado profesional.</t>
         </is>
       </c>
       <c r="E62" s="219" t="n">
-        <v>2831</v>
+        <v>8424</v>
       </c>
       <c r="F62" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G62" s="217" t="inlineStr">
@@ -5803,16 +5803,16 @@
       </c>
       <c r="C63" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Peinado Novia Individual</t>
+          <t>Andrea Lozano - Maquillaje Aerógrafo Novia Ind</t>
         </is>
       </c>
       <c r="D63" s="218" t="inlineStr">
         <is>
-          <t>Peinado de novia individual con colocación de tocado y velo.</t>
+          <t>Maquillaje aerógrafo individual para novia/quinceañera.</t>
         </is>
       </c>
       <c r="E63" s="219" t="n">
-        <v>2457</v>
+        <v>2960</v>
       </c>
       <c r="F63" s="220" t="inlineStr">
         <is>
@@ -5841,16 +5841,16 @@
       </c>
       <c r="C64" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Peinado + Aero Invitadas</t>
+          <t>Andrea Lozano - Maquillaje Tradicional Novia Ind</t>
         </is>
       </c>
       <c r="D64" s="218" t="inlineStr">
         <is>
-          <t>Servicio a domicilio de peinado y maquillaje aerógrafo para acompañantes.</t>
+          <t>Maquillaje tradicional individual para novia/quinceañera.</t>
         </is>
       </c>
       <c r="E64" s="219" t="n">
-        <v>2867</v>
+        <v>2831</v>
       </c>
       <c r="F64" s="220" t="inlineStr">
         <is>
@@ -5879,16 +5879,16 @@
       </c>
       <c r="C65" s="218" t="inlineStr">
         <is>
-          <t>Andrea Lozano - Peinado + Tradicional Invitadas</t>
+          <t>Andrea Lozano - Peinado Novia Individual</t>
         </is>
       </c>
       <c r="D65" s="218" t="inlineStr">
         <is>
-          <t>Servicio a domicilio de peinado y maquillaje tradicional para acompañantes.</t>
+          <t>Peinado de novia individual con colocación de tocado y velo.</t>
         </is>
       </c>
       <c r="E65" s="219" t="n">
-        <v>2574</v>
+        <v>2457</v>
       </c>
       <c r="F65" s="220" t="inlineStr">
         <is>
@@ -5917,16 +5917,16 @@
       </c>
       <c r="C66" s="218" t="inlineStr">
         <is>
-          <t>Barbero (novio)</t>
+          <t>Andrea Lozano - Peinado + Aero Invitadas</t>
         </is>
       </c>
       <c r="D66" s="218" t="inlineStr">
         <is>
-          <t>Corte y arreglo de barba profesional para el novio el gran día.</t>
+          <t>Servicio a domicilio de peinado y maquillaje aerógrafo para acompañantes.</t>
         </is>
       </c>
       <c r="E66" s="219" t="n">
-        <v>800</v>
+        <v>2867</v>
       </c>
       <c r="F66" s="220" t="inlineStr">
         <is>
@@ -5938,7 +5938,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H66" s="218" t="inlineStr"/>
+      <c r="H66" s="218">
+        <f>HYPERLINK("https://wa.me/527774587923","Pedir Andrea Lozano")</f>
+        <v/>
+      </c>
       <c r="I66" s="216" t="n"/>
     </row>
     <row r="67" ht="18" customHeight="1" s="107">
@@ -5952,16 +5955,16 @@
       </c>
       <c r="C67" s="218" t="inlineStr">
         <is>
-          <t>Spa / Tratamientos previos</t>
+          <t>Andrea Lozano - Peinado + Tradicional Invitadas</t>
         </is>
       </c>
       <c r="D67" s="218" t="inlineStr">
         <is>
-          <t>Sesiones faciales y de relajación pre-boda.</t>
+          <t>Servicio a domicilio de peinado y maquillaje tradicional para acompañantes.</t>
         </is>
       </c>
       <c r="E67" s="219" t="n">
-        <v>2500</v>
+        <v>2574</v>
       </c>
       <c r="F67" s="220" t="inlineStr">
         <is>
@@ -5973,49 +5976,72 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H67" s="218" t="inlineStr"/>
+      <c r="H67" s="218">
+        <f>HYPERLINK("https://wa.me/527774587923","Pedir Andrea Lozano")</f>
+        <v/>
+      </c>
       <c r="I67" s="216" t="n"/>
     </row>
     <row r="68" ht="18" customHeight="1" s="107">
-      <c r="A68" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Vestuario</t>
-        </is>
-      </c>
-      <c r="B68" s="216" t="n"/>
-      <c r="C68" s="216" t="n"/>
-      <c r="D68" s="216" t="n"/>
-      <c r="E68" s="216" t="n"/>
-      <c r="F68" s="216" t="n"/>
-      <c r="G68" s="216" t="n"/>
-      <c r="H68" s="216" t="n"/>
+      <c r="A68" s="217" t="n">
+        <v>60</v>
+      </c>
+      <c r="B68" s="218" t="inlineStr">
+        <is>
+          <t>Belleza &amp; Imagen</t>
+        </is>
+      </c>
+      <c r="C68" s="218" t="inlineStr">
+        <is>
+          <t>Barbero (novio)</t>
+        </is>
+      </c>
+      <c r="D68" s="218" t="inlineStr">
+        <is>
+          <t>Corte y arreglo de barba profesional para el novio el gran día.</t>
+        </is>
+      </c>
+      <c r="E68" s="219" t="n">
+        <v>800</v>
+      </c>
+      <c r="F68" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G68" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H68" s="218" t="inlineStr"/>
       <c r="I68" s="216" t="n"/>
     </row>
     <row r="69" ht="18" customHeight="1" s="107">
       <c r="A69" s="217" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B69" s="218" t="inlineStr">
         <is>
-          <t>Vestuario</t>
+          <t>Belleza &amp; Imagen</t>
         </is>
       </c>
       <c r="C69" s="218" t="inlineStr">
         <is>
-          <t>Vestido de novia / XV</t>
+          <t>Spa / Tratamientos previos</t>
         </is>
       </c>
       <c r="D69" s="218" t="inlineStr">
         <is>
-          <t>Vestido de gala principal seleccionado.</t>
+          <t>Sesiones faciales y de relajación pre-boda.</t>
         </is>
       </c>
       <c r="E69" s="219" t="n">
-        <v>18000</v>
+        <v>2500</v>
       </c>
       <c r="F69" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G69" s="217" t="inlineStr">
@@ -6027,38 +6053,18 @@
       <c r="I69" s="216" t="n"/>
     </row>
     <row r="70" ht="18" customHeight="1" s="107">
-      <c r="A70" s="217" t="n">
-        <v>61</v>
-      </c>
-      <c r="B70" s="218" t="inlineStr">
-        <is>
-          <t>Vestuario</t>
-        </is>
-      </c>
-      <c r="C70" s="218" t="inlineStr">
-        <is>
-          <t>Traje del novio</t>
-        </is>
-      </c>
-      <c r="D70" s="218" t="inlineStr">
-        <is>
-          <t>Traje sastre o smoking premium.</t>
-        </is>
-      </c>
-      <c r="E70" s="219" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F70" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G70" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H70" s="218" t="inlineStr"/>
+      <c r="A70" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vestuario</t>
+        </is>
+      </c>
+      <c r="B70" s="216" t="n"/>
+      <c r="C70" s="216" t="n"/>
+      <c r="D70" s="216" t="n"/>
+      <c r="E70" s="216" t="n"/>
+      <c r="F70" s="216" t="n"/>
+      <c r="G70" s="216" t="n"/>
+      <c r="H70" s="216" t="n"/>
       <c r="I70" s="216" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1" s="107">
@@ -6072,20 +6078,20 @@
       </c>
       <c r="C71" s="218" t="inlineStr">
         <is>
-          <t>Vestidos de damas</t>
+          <t>Vestido de novia / XV</t>
         </is>
       </c>
       <c r="D71" s="218" t="inlineStr">
         <is>
-          <t>Lote de vestidos para las damas de honor.</t>
+          <t>Vestido de gala principal seleccionado.</t>
         </is>
       </c>
       <c r="E71" s="219" t="n">
-        <v>7500</v>
+        <v>18000</v>
       </c>
       <c r="F71" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G71" s="217" t="inlineStr">
@@ -6107,20 +6113,20 @@
       </c>
       <c r="C72" s="218" t="inlineStr">
         <is>
-          <t>Renta de smoking</t>
+          <t>Traje del novio</t>
         </is>
       </c>
       <c r="D72" s="218" t="inlineStr">
         <is>
-          <t>Smoking para los chambelanes o familiares.</t>
+          <t>Traje sastre o smoking premium.</t>
         </is>
       </c>
       <c r="E72" s="219" t="n">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="F72" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G72" s="217" t="inlineStr">
@@ -6142,16 +6148,16 @@
       </c>
       <c r="C73" s="218" t="inlineStr">
         <is>
-          <t>Accesorios (velo, tiara, etc.)</t>
+          <t>Vestidos de damas</t>
         </is>
       </c>
       <c r="D73" s="218" t="inlineStr">
         <is>
-          <t>Accesorios de novia/quinceañera.</t>
+          <t>Lote de vestidos para las damas de honor.</t>
         </is>
       </c>
       <c r="E73" s="219" t="n">
-        <v>2500</v>
+        <v>7500</v>
       </c>
       <c r="F73" s="220" t="inlineStr">
         <is>
@@ -6177,16 +6183,16 @@
       </c>
       <c r="C74" s="218" t="inlineStr">
         <is>
-          <t>Zapatos</t>
+          <t>Renta de smoking</t>
         </is>
       </c>
       <c r="D74" s="218" t="inlineStr">
         <is>
-          <t>Calzado especial cómodo y de gala.</t>
+          <t>Smoking para los chambelanes o familiares.</t>
         </is>
       </c>
       <c r="E74" s="219" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="F74" s="220" t="inlineStr">
         <is>
@@ -6202,45 +6208,65 @@
       <c r="I74" s="216" t="n"/>
     </row>
     <row r="75" ht="18" customHeight="1" s="107">
-      <c r="A75" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Coreografia &amp; Show</t>
-        </is>
-      </c>
-      <c r="B75" s="216" t="n"/>
-      <c r="C75" s="216" t="n"/>
-      <c r="D75" s="216" t="n"/>
-      <c r="E75" s="216" t="n"/>
-      <c r="F75" s="216" t="n"/>
-      <c r="G75" s="216" t="n"/>
-      <c r="H75" s="216" t="n"/>
+      <c r="A75" s="217" t="n">
+        <v>66</v>
+      </c>
+      <c r="B75" s="218" t="inlineStr">
+        <is>
+          <t>Vestuario</t>
+        </is>
+      </c>
+      <c r="C75" s="218" t="inlineStr">
+        <is>
+          <t>Accesorios (velo, tiara, etc.)</t>
+        </is>
+      </c>
+      <c r="D75" s="218" t="inlineStr">
+        <is>
+          <t>Accesorios de novia/quinceañera.</t>
+        </is>
+      </c>
+      <c r="E75" s="219" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F75" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G75" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H75" s="218" t="inlineStr"/>
       <c r="I75" s="216" t="n"/>
     </row>
     <row r="76" ht="19.5" customHeight="1" s="107">
       <c r="A76" s="217" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B76" s="218" t="inlineStr">
         <is>
-          <t>Coreografia &amp; Show</t>
+          <t>Vestuario</t>
         </is>
       </c>
       <c r="C76" s="218" t="inlineStr">
         <is>
-          <t>Dance Queens - Paquete Vals Básico</t>
+          <t>Zapatos</t>
         </is>
       </c>
       <c r="D76" s="218" t="inlineStr">
         <is>
-          <t>Coreografía oficial del vals, 6 clases de ensayo y copas decoradas de regalo.</t>
+          <t>Calzado especial cómodo y de gala.</t>
         </is>
       </c>
       <c r="E76" s="219" t="n">
-        <v>7605</v>
+        <v>2000</v>
       </c>
       <c r="F76" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G76" s="217" t="inlineStr">
@@ -6248,48 +6274,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H76" s="218">
-        <f>HYPERLINK("https://wa.me/527772994425","Pedir Dance Queens")</f>
-        <v/>
-      </c>
+      <c r="H76" s="218" t="inlineStr"/>
       <c r="I76" s="216" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1" s="107">
-      <c r="A77" s="217" t="n">
-        <v>67</v>
-      </c>
-      <c r="B77" s="218" t="inlineStr">
-        <is>
-          <t>Coreografia &amp; Show</t>
-        </is>
-      </c>
-      <c r="C77" s="218" t="inlineStr">
-        <is>
-          <t>Dance Queens - Paquete Vals VIP</t>
-        </is>
-      </c>
-      <c r="D77" s="218" t="inlineStr">
-        <is>
-          <t>Coreografía Vals, moderna y show con pirotecnia fría e hidrogel led (10 clases).</t>
-        </is>
-      </c>
-      <c r="E77" s="219" t="n">
-        <v>11115</v>
-      </c>
-      <c r="F77" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G77" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H77" s="218">
-        <f>HYPERLINK("https://wa.me/527772994425","Pedir Dance Queens")</f>
-        <v/>
-      </c>
+      <c r="A77" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Coreografia &amp; Show</t>
+        </is>
+      </c>
+      <c r="B77" s="216" t="n"/>
+      <c r="C77" s="216" t="n"/>
+      <c r="D77" s="216" t="n"/>
+      <c r="E77" s="216" t="n"/>
+      <c r="F77" s="216" t="n"/>
+      <c r="G77" s="216" t="n"/>
+      <c r="H77" s="216" t="n"/>
       <c r="I77" s="216" t="n"/>
     </row>
     <row r="78" ht="18" customHeight="1" s="107">
@@ -6303,16 +6303,16 @@
       </c>
       <c r="C78" s="218" t="inlineStr">
         <is>
-          <t>Ensayos grupales extras</t>
+          <t>Dance Queens - Paquete Vals Básico</t>
         </is>
       </c>
       <c r="D78" s="218" t="inlineStr">
         <is>
-          <t>Clases adicionales para repasar pasos y sincronización.</t>
+          <t>Coreografía oficial del vals, 6 clases de ensayo y copas decoradas de regalo.</t>
         </is>
       </c>
       <c r="E78" s="219" t="n">
-        <v>1500</v>
+        <v>7605</v>
       </c>
       <c r="F78" s="220" t="inlineStr">
         <is>
@@ -6324,45 +6324,71 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H78" s="218" t="inlineStr"/>
+      <c r="H78" s="218">
+        <f>HYPERLINK("https://wa.me/527772994425","Pedir Dance Queens")</f>
+        <v/>
+      </c>
       <c r="I78" s="216" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1" s="107">
-      <c r="A79" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Decoracion &amp; Diseno</t>
-        </is>
-      </c>
-      <c r="B79" s="216" t="n"/>
-      <c r="C79" s="216" t="n"/>
-      <c r="D79" s="216" t="n"/>
-      <c r="E79" s="216" t="n"/>
-      <c r="F79" s="216" t="n"/>
-      <c r="G79" s="216" t="n"/>
-      <c r="H79" s="216" t="n"/>
+      <c r="A79" s="217" t="n">
+        <v>69</v>
+      </c>
+      <c r="B79" s="218" t="inlineStr">
+        <is>
+          <t>Coreografia &amp; Show</t>
+        </is>
+      </c>
+      <c r="C79" s="218" t="inlineStr">
+        <is>
+          <t>Dance Queens - Paquete Vals VIP</t>
+        </is>
+      </c>
+      <c r="D79" s="218" t="inlineStr">
+        <is>
+          <t>Coreografía Vals, moderna y show con pirotecnia fría e hidrogel led (10 clases).</t>
+        </is>
+      </c>
+      <c r="E79" s="219" t="n">
+        <v>11115</v>
+      </c>
+      <c r="F79" s="220" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G79" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="218">
+        <f>HYPERLINK("https://wa.me/527772994425","Pedir Dance Queens")</f>
+        <v/>
+      </c>
       <c r="I79" s="216" t="n"/>
     </row>
     <row r="80" ht="18" customHeight="1" s="107">
       <c r="A80" s="217" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B80" s="218" t="inlineStr">
         <is>
-          <t>Decoracion &amp; Diseno</t>
+          <t>Coreografia &amp; Show</t>
         </is>
       </c>
       <c r="C80" s="218" t="inlineStr">
         <is>
-          <t>Jessy &amp; Richard - Coordinación Básica</t>
+          <t>Ensayos grupales extras</t>
         </is>
       </c>
       <c r="D80" s="218" t="inlineStr">
         <is>
-          <t>Planificación inicial de presupuesto, proveedores y timing de la boda.</t>
+          <t>Clases adicionales para repasar pasos y sincronización.</t>
         </is>
       </c>
       <c r="E80" s="219" t="n">
-        <v>17550</v>
+        <v>1500</v>
       </c>
       <c r="F80" s="220" t="inlineStr">
         <is>
@@ -6374,48 +6400,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H80" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Jessy &amp; Richard")</f>
-        <v/>
-      </c>
+      <c r="H80" s="218" t="inlineStr"/>
       <c r="I80" s="216" t="n"/>
     </row>
     <row r="81" ht="18" customHeight="1" s="107">
-      <c r="A81" s="217" t="n">
-        <v>70</v>
-      </c>
-      <c r="B81" s="218" t="inlineStr">
-        <is>
-          <t>Decoracion &amp; Diseno</t>
-        </is>
-      </c>
-      <c r="C81" s="218" t="inlineStr">
-        <is>
-          <t>Jessy &amp; Richard - Coordinación Full VIP</t>
-        </is>
-      </c>
-      <c r="D81" s="218" t="inlineStr">
-        <is>
-          <t>Coordinación y producción total de inicio a fin del evento en la locación.</t>
-        </is>
-      </c>
-      <c r="E81" s="219" t="n">
-        <v>35100</v>
-      </c>
-      <c r="F81" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G81" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H81" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Jessy &amp; Richard")</f>
-        <v/>
-      </c>
+      <c r="A81" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Decoracion &amp; Diseno</t>
+        </is>
+      </c>
+      <c r="B81" s="216" t="n"/>
+      <c r="C81" s="216" t="n"/>
+      <c r="D81" s="216" t="n"/>
+      <c r="E81" s="216" t="n"/>
+      <c r="F81" s="216" t="n"/>
+      <c r="G81" s="216" t="n"/>
+      <c r="H81" s="216" t="n"/>
       <c r="I81" s="216" t="n"/>
     </row>
     <row r="82" ht="19.5" customHeight="1" s="107">
@@ -6429,16 +6429,16 @@
       </c>
       <c r="C82" s="218" t="inlineStr">
         <is>
-          <t>Kataleya Florist - Ramo de Novia Premium</t>
+          <t>Jessy &amp; Richard - Coordinación Básica</t>
         </is>
       </c>
       <c r="D82" s="218" t="inlineStr">
         <is>
-          <t>Arreglo floral exclusivo con flores de gala importadas y orquídeas.</t>
+          <t>Planificación inicial de presupuesto, proveedores y timing de la boda.</t>
         </is>
       </c>
       <c r="E82" s="219" t="n">
-        <v>32760</v>
+        <v>17550</v>
       </c>
       <c r="F82" s="220" t="inlineStr">
         <is>
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="H82" s="218">
-        <f>HYPERLINK("https://wa.me/527775114425","Pedir Kataleya")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Jessy &amp; Richard")</f>
         <v/>
       </c>
       <c r="I82" s="216" t="n"/>
@@ -6467,16 +6467,16 @@
       </c>
       <c r="C83" s="218" t="inlineStr">
         <is>
-          <t>Kataleya Florist - Centros de Mesa Gala</t>
+          <t>Jessy &amp; Richard - Coordinación Full VIP</t>
         </is>
       </c>
       <c r="D83" s="218" t="inlineStr">
         <is>
-          <t>Arreglos florales frescos de altura para mesas de comensales.</t>
+          <t>Coordinación y producción total de inicio a fin del evento en la locación.</t>
         </is>
       </c>
       <c r="E83" s="219" t="n">
-        <v>995</v>
+        <v>35100</v>
       </c>
       <c r="F83" s="220" t="inlineStr">
         <is>
@@ -6489,7 +6489,7 @@
         </is>
       </c>
       <c r="H83" s="218">
-        <f>HYPERLINK("https://wa.me/527775114425","Pedir Kataleya")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Jessy &amp; Richard")</f>
         <v/>
       </c>
       <c r="I83" s="216" t="n"/>
@@ -6505,16 +6505,16 @@
       </c>
       <c r="C84" s="218" t="inlineStr">
         <is>
-          <t>Kataleya Florist - Decoración de Altar/Ceremonia</t>
+          <t>Kataleya Florist - Ramo de Novia Premium</t>
         </is>
       </c>
       <c r="D84" s="218" t="inlineStr">
         <is>
-          <t>Set de flores de gala y decoración para pasillo y altar.</t>
+          <t>Arreglo floral exclusivo con flores de gala importadas y orquídeas.</t>
         </is>
       </c>
       <c r="E84" s="219" t="n">
-        <v>8775</v>
+        <v>32760</v>
       </c>
       <c r="F84" s="220" t="inlineStr">
         <is>
@@ -6543,20 +6543,20 @@
       </c>
       <c r="C85" s="218" t="inlineStr">
         <is>
-          <t>Aby Decora - Bouquet 15 Años</t>
+          <t>Kataleya Florist - Centros de Mesa Gala</t>
         </is>
       </c>
       <c r="D85" s="218" t="inlineStr">
         <is>
-          <t>Montaje decorativo de globos con número gigante de 15 años.</t>
+          <t>Arreglos florales frescos de altura para mesas de comensales.</t>
         </is>
       </c>
       <c r="E85" s="219" t="n">
-        <v>2925</v>
+        <v>995</v>
       </c>
       <c r="F85" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G85" s="217" t="inlineStr">
@@ -6565,7 +6565,7 @@
         </is>
       </c>
       <c r="H85" s="218">
-        <f>HYPERLINK("https://wa.me/527774587923","Pedir Aby Decora")</f>
+        <f>HYPERLINK("https://wa.me/527775114425","Pedir Kataleya")</f>
         <v/>
       </c>
       <c r="I85" s="216" t="n"/>
@@ -6581,20 +6581,20 @@
       </c>
       <c r="C86" s="218" t="inlineStr">
         <is>
-          <t>Aby Decora - Montaje Arco Globos</t>
+          <t>Kataleya Florist - Decoración de Altar/Ceremonia</t>
         </is>
       </c>
       <c r="D86" s="218" t="inlineStr">
         <is>
-          <t>Arco orgánico de globos premium para entrada o mesa de honor.</t>
+          <t>Set de flores de gala y decoración para pasillo y altar.</t>
         </is>
       </c>
       <c r="E86" s="219" t="n">
-        <v>3510</v>
+        <v>8775</v>
       </c>
       <c r="F86" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G86" s="217" t="inlineStr">
@@ -6603,7 +6603,7 @@
         </is>
       </c>
       <c r="H86" s="218">
-        <f>HYPERLINK("https://wa.me/527774587923","Pedir Aby Decora")</f>
+        <f>HYPERLINK("https://wa.me/527775114425","Pedir Kataleya")</f>
         <v/>
       </c>
       <c r="I86" s="216" t="n"/>
@@ -6619,16 +6619,16 @@
       </c>
       <c r="C87" s="218" t="inlineStr">
         <is>
-          <t>Aby Decora - Panel Back Globos</t>
+          <t>Aby Decora - Bouquet 15 Años</t>
         </is>
       </c>
       <c r="D87" s="218" t="inlineStr">
         <is>
-          <t>Panel circular con set de globos y luces de neón decorativas.</t>
+          <t>Montaje decorativo de globos con número gigante de 15 años.</t>
         </is>
       </c>
       <c r="E87" s="219" t="n">
-        <v>5265</v>
+        <v>2925</v>
       </c>
       <c r="F87" s="220" t="inlineStr">
         <is>
@@ -6657,16 +6657,16 @@
       </c>
       <c r="C88" s="218" t="inlineStr">
         <is>
-          <t>Aby Decora - Decoración Total Globos</t>
+          <t>Aby Decora - Montaje Arco Globos</t>
         </is>
       </c>
       <c r="D88" s="218" t="inlineStr">
         <is>
-          <t>Decoración total: Mesa de honor, mesa de dulces, back y entrada.</t>
+          <t>Arco orgánico de globos premium para entrada o mesa de honor.</t>
         </is>
       </c>
       <c r="E88" s="219" t="n">
-        <v>5850</v>
+        <v>3510</v>
       </c>
       <c r="F88" s="220" t="inlineStr">
         <is>
@@ -6695,16 +6695,16 @@
       </c>
       <c r="C89" s="218" t="inlineStr">
         <is>
-          <t>Mobiliario temático</t>
+          <t>Aby Decora - Panel Back Globos</t>
         </is>
       </c>
       <c r="D89" s="218" t="inlineStr">
         <is>
-          <t>Renta de mesas de madera, sillas crossback o salas lounge.</t>
+          <t>Panel circular con set de globos y luces de neón decorativas.</t>
         </is>
       </c>
       <c r="E89" s="219" t="n">
-        <v>4500</v>
+        <v>5265</v>
       </c>
       <c r="F89" s="220" t="inlineStr">
         <is>
@@ -6716,7 +6716,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H89" s="218" t="inlineStr"/>
+      <c r="H89" s="218">
+        <f>HYPERLINK("https://wa.me/527774587923","Pedir Aby Decora")</f>
+        <v/>
+      </c>
       <c r="I89" s="216" t="n"/>
     </row>
     <row r="90" ht="19.5" customHeight="1" s="107">
@@ -6730,16 +6733,16 @@
       </c>
       <c r="C90" s="218" t="inlineStr">
         <is>
-          <t>Mantelería premium</t>
+          <t>Aby Decora - Decoración Total Globos</t>
         </is>
       </c>
       <c r="D90" s="218" t="inlineStr">
         <is>
-          <t>Manteles de gala, caminos de mesa y servilletas bordadas.</t>
+          <t>Decoración total: Mesa de honor, mesa de dulces, back y entrada.</t>
         </is>
       </c>
       <c r="E90" s="219" t="n">
-        <v>2500</v>
+        <v>5850</v>
       </c>
       <c r="F90" s="220" t="inlineStr">
         <is>
@@ -6751,45 +6754,68 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H90" s="218" t="inlineStr"/>
+      <c r="H90" s="218">
+        <f>HYPERLINK("https://wa.me/527774587923","Pedir Aby Decora")</f>
+        <v/>
+      </c>
       <c r="I90" s="216" t="n"/>
     </row>
     <row r="91" ht="18" customHeight="1" s="107">
-      <c r="A91" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Produccion &amp; Montaje</t>
-        </is>
-      </c>
-      <c r="B91" s="216" t="n"/>
-      <c r="C91" s="216" t="n"/>
-      <c r="D91" s="216" t="n"/>
-      <c r="E91" s="216" t="n"/>
-      <c r="F91" s="216" t="n"/>
-      <c r="G91" s="216" t="n"/>
-      <c r="H91" s="216" t="n"/>
+      <c r="A91" s="217" t="n">
+        <v>80</v>
+      </c>
+      <c r="B91" s="218" t="inlineStr">
+        <is>
+          <t>Decoracion &amp; Diseno</t>
+        </is>
+      </c>
+      <c r="C91" s="218" t="inlineStr">
+        <is>
+          <t>Mobiliario temático</t>
+        </is>
+      </c>
+      <c r="D91" s="218" t="inlineStr">
+        <is>
+          <t>Renta de mesas de madera, sillas crossback o salas lounge.</t>
+        </is>
+      </c>
+      <c r="E91" s="219" t="n">
+        <v>4500</v>
+      </c>
+      <c r="F91" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G91" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="218" t="inlineStr"/>
       <c r="I91" s="216" t="n"/>
     </row>
     <row r="92" ht="18" customHeight="1" s="107">
       <c r="A92" s="217" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B92" s="218" t="inlineStr">
         <is>
-          <t>Produccion &amp; Montaje</t>
+          <t>Decoracion &amp; Diseno</t>
         </is>
       </c>
       <c r="C92" s="218" t="inlineStr">
         <is>
-          <t>Proveedor de Pantallas - LED P3 (3x2m)</t>
+          <t>Mantelería premium</t>
         </is>
       </c>
       <c r="D92" s="218" t="inlineStr">
         <is>
-          <t>Pantalla gigante de alta definición con soporte, cableado y operador.</t>
+          <t>Manteles de gala, caminos de mesa y servilletas bordadas.</t>
         </is>
       </c>
       <c r="E92" s="219" t="n">
-        <v>9945</v>
+        <v>2500</v>
       </c>
       <c r="F92" s="220" t="inlineStr">
         <is>
@@ -6801,48 +6827,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H92" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/","Ver Proveedor Pantallas")</f>
-        <v/>
-      </c>
+      <c r="H92" s="218" t="inlineStr"/>
       <c r="I92" s="216" t="n"/>
     </row>
     <row r="93" ht="18" customHeight="1" s="107">
-      <c r="A93" s="217" t="n">
-        <v>81</v>
-      </c>
-      <c r="B93" s="218" t="inlineStr">
-        <is>
-          <t>Produccion &amp; Montaje</t>
-        </is>
-      </c>
-      <c r="C93" s="218" t="inlineStr">
-        <is>
-          <t>Proveedor de Pantallas - LED P3 (4x3m)</t>
-        </is>
-      </c>
-      <c r="D93" s="218" t="inlineStr">
-        <is>
-          <t>Pantalla gigante LED P3 premium de gran alcance con operador.</t>
-        </is>
-      </c>
-      <c r="E93" s="219" t="n">
-        <v>14040</v>
-      </c>
-      <c r="F93" s="220" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G93" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H93" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/","Ver Proveedor Pantallas")</f>
-        <v/>
-      </c>
+      <c r="A93" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Produccion &amp; Montaje</t>
+        </is>
+      </c>
+      <c r="B93" s="216" t="n"/>
+      <c r="C93" s="216" t="n"/>
+      <c r="D93" s="216" t="n"/>
+      <c r="E93" s="216" t="n"/>
+      <c r="F93" s="216" t="n"/>
+      <c r="G93" s="216" t="n"/>
+      <c r="H93" s="216" t="n"/>
       <c r="I93" s="216" t="n"/>
     </row>
     <row r="94" ht="18" customHeight="1" s="107">
@@ -6856,20 +6856,20 @@
       </c>
       <c r="C94" s="218" t="inlineStr">
         <is>
-          <t>Iluminación arquitectónica</t>
+          <t>Proveedor de Pantallas - LED P3 (3x2m)</t>
         </is>
       </c>
       <c r="D94" s="218" t="inlineStr">
         <is>
-          <t>Montaje de luces ambientales en columnas y áreas clave del salón.</t>
+          <t>Pantalla gigante de alta definición con soporte, cableado y operador.</t>
         </is>
       </c>
       <c r="E94" s="219" t="n">
-        <v>6000</v>
+        <v>9945</v>
       </c>
       <c r="F94" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G94" s="217" t="inlineStr">
@@ -6877,7 +6877,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H94" s="218" t="inlineStr"/>
+      <c r="H94" s="218">
+        <f>HYPERLINK("https://primaveraeventsgroup.com/","Ver Proveedor Pantallas")</f>
+        <v/>
+      </c>
       <c r="I94" s="216" t="n"/>
     </row>
     <row r="95" ht="19.5" customHeight="1" s="107">
@@ -6891,20 +6894,20 @@
       </c>
       <c r="C95" s="218" t="inlineStr">
         <is>
-          <t>Audio profesional</t>
+          <t>Proveedor de Pantallas - LED P3 (4x3m)</t>
         </is>
       </c>
       <c r="D95" s="218" t="inlineStr">
         <is>
-          <t>Equipamiento de bocinas line array de alta fidelidad para el banquete.</t>
+          <t>Pantalla gigante LED P3 premium de gran alcance con operador.</t>
         </is>
       </c>
       <c r="E95" s="219" t="n">
-        <v>5000</v>
+        <v>14040</v>
       </c>
       <c r="F95" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G95" s="217" t="inlineStr">
@@ -6912,7 +6915,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H95" s="218" t="inlineStr"/>
+      <c r="H95" s="218">
+        <f>HYPERLINK("https://primaveraeventsgroup.com/","Ver Proveedor Pantallas")</f>
+        <v/>
+      </c>
       <c r="I95" s="216" t="n"/>
     </row>
     <row r="96" ht="18" customHeight="1" s="107">
@@ -6926,20 +6932,20 @@
       </c>
       <c r="C96" s="218" t="inlineStr">
         <is>
-          <t>Estructuras / Tarimas</t>
+          <t>Iluminación arquitectónica</t>
         </is>
       </c>
       <c r="D96" s="218" t="inlineStr">
         <is>
-          <t>Montaje de pista y estructuras de aluminio elevadas para luces.</t>
+          <t>Montaje de luces ambientales en columnas y áreas clave del salón.</t>
         </is>
       </c>
       <c r="E96" s="219" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="F96" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G96" s="217" t="inlineStr">
@@ -6951,45 +6957,65 @@
       <c r="I96" s="216" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1" s="107">
-      <c r="A97" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Papeleria &amp; Diseno Grafico</t>
-        </is>
-      </c>
-      <c r="B97" s="216" t="n"/>
-      <c r="C97" s="216" t="n"/>
-      <c r="D97" s="216" t="n"/>
-      <c r="E97" s="216" t="n"/>
-      <c r="F97" s="216" t="n"/>
-      <c r="G97" s="216" t="n"/>
-      <c r="H97" s="216" t="n"/>
+      <c r="A97" s="217" t="n">
+        <v>85</v>
+      </c>
+      <c r="B97" s="218" t="inlineStr">
+        <is>
+          <t>Produccion &amp; Montaje</t>
+        </is>
+      </c>
+      <c r="C97" s="218" t="inlineStr">
+        <is>
+          <t>Audio profesional</t>
+        </is>
+      </c>
+      <c r="D97" s="218" t="inlineStr">
+        <is>
+          <t>Equipamiento de bocinas line array de alta fidelidad para el banquete.</t>
+        </is>
+      </c>
+      <c r="E97" s="219" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F97" s="220" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G97" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" s="218" t="inlineStr"/>
       <c r="I97" s="216" t="n"/>
     </row>
     <row r="98" ht="18" customHeight="1" s="107">
       <c r="A98" s="217" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B98" s="218" t="inlineStr">
         <is>
-          <t>Papeleria &amp; Diseno Grafico</t>
+          <t>Produccion &amp; Montaje</t>
         </is>
       </c>
       <c r="C98" s="218" t="inlineStr">
         <is>
-          <t>INIT Idea - Invitación Digital Premium</t>
+          <t>Estructuras / Tarimas</t>
         </is>
       </c>
       <c r="D98" s="218" t="inlineStr">
         <is>
-          <t>Invitación interactiva con música, confirmación, mapa y cronograma.</t>
+          <t>Montaje de pista y estructuras de aluminio elevadas para luces.</t>
         </is>
       </c>
       <c r="E98" s="219" t="n">
-        <v>1755</v>
+        <v>5000</v>
       </c>
       <c r="F98" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G98" s="217" t="inlineStr">
@@ -6997,48 +7023,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H98" s="218">
-        <f>HYPERLINK("https://5410m0n0c001.github.io/INIT-IDEA/invitaciones.html","Ver INIT Idea")</f>
-        <v/>
-      </c>
+      <c r="H98" s="218" t="inlineStr"/>
       <c r="I98" s="216" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1" s="107">
-      <c r="A99" s="217" t="n">
-        <v>86</v>
-      </c>
-      <c r="B99" s="218" t="inlineStr">
-        <is>
-          <t>Papeleria &amp; Diseno Grafico</t>
-        </is>
-      </c>
-      <c r="C99" s="218" t="inlineStr">
-        <is>
-          <t>INIT Idea - Invitación Digital VIP</t>
-        </is>
-      </c>
-      <c r="D99" s="218" t="inlineStr">
-        <is>
-          <t>Invitación interactiva con pases QR individuales, confirmación y RSVP.</t>
-        </is>
-      </c>
-      <c r="E99" s="219" t="n">
-        <v>2925</v>
-      </c>
-      <c r="F99" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G99" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H99" s="218">
-        <f>HYPERLINK("https://5410m0n0c001.github.io/INIT-IDEA/invitaciones.html","Ver INIT Idea")</f>
-        <v/>
-      </c>
+      <c r="A99" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Papeleria &amp; Diseno Grafico</t>
+        </is>
+      </c>
+      <c r="B99" s="216" t="n"/>
+      <c r="C99" s="216" t="n"/>
+      <c r="D99" s="216" t="n"/>
+      <c r="E99" s="216" t="n"/>
+      <c r="F99" s="216" t="n"/>
+      <c r="G99" s="216" t="n"/>
+      <c r="H99" s="216" t="n"/>
       <c r="I99" s="216" t="n"/>
     </row>
     <row r="100" ht="18" customHeight="1" s="107">
@@ -7052,16 +7052,16 @@
       </c>
       <c r="C100" s="218" t="inlineStr">
         <is>
-          <t>Invitaciones físicas</t>
+          <t>INIT Idea - Invitación Digital Premium</t>
         </is>
       </c>
       <c r="D100" s="218" t="inlineStr">
         <is>
-          <t>Invitaciones impresas en papel fino y sobres personalizados.</t>
+          <t>Invitación interactiva con música, confirmación, mapa y cronograma.</t>
         </is>
       </c>
       <c r="E100" s="219" t="n">
-        <v>3500</v>
+        <v>1755</v>
       </c>
       <c r="F100" s="220" t="inlineStr">
         <is>
@@ -7073,7 +7073,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H100" s="218" t="inlineStr"/>
+      <c r="H100" s="218">
+        <f>HYPERLINK("https://5410m0n0c001.github.io/INIT-IDEA/invitaciones.html","Ver INIT Idea")</f>
+        <v/>
+      </c>
       <c r="I100" s="216" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1" s="107">
@@ -7087,20 +7090,20 @@
       </c>
       <c r="C101" s="218" t="inlineStr">
         <is>
-          <t>Save the date digital</t>
+          <t>INIT Idea - Invitación Digital VIP</t>
         </is>
       </c>
       <c r="D101" s="218" t="inlineStr">
         <is>
-          <t>Folleto digital para anticipar la fecha en redes.</t>
+          <t>Invitación interactiva con pases QR individuales, confirmación y RSVP.</t>
         </is>
       </c>
       <c r="E101" s="219" t="n">
-        <v>1200</v>
+        <v>2925</v>
       </c>
       <c r="F101" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G101" s="217" t="inlineStr">
@@ -7108,7 +7111,10 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H101" s="218" t="inlineStr"/>
+      <c r="H101" s="218">
+        <f>HYPERLINK("https://5410m0n0c001.github.io/INIT-IDEA/invitaciones.html","Ver INIT Idea")</f>
+        <v/>
+      </c>
       <c r="I101" s="216" t="n"/>
     </row>
     <row r="102" ht="19.5" customHeight="1" s="107">
@@ -7122,20 +7128,20 @@
       </c>
       <c r="C102" s="218" t="inlineStr">
         <is>
-          <t>Menús impresos</t>
+          <t>Invitaciones físicas</t>
         </is>
       </c>
       <c r="D102" s="218" t="inlineStr">
         <is>
-          <t>Minutas del menú por persona en cada lugar de mesa.</t>
+          <t>Invitaciones impresas en papel fino y sobres personalizados.</t>
         </is>
       </c>
       <c r="E102" s="219" t="n">
-        <v>800</v>
+        <v>3500</v>
       </c>
       <c r="F102" s="220" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G102" s="217" t="inlineStr">
@@ -7147,45 +7153,65 @@
       <c r="I102" s="216" t="n"/>
     </row>
     <row r="103" ht="18" customHeight="1" s="107">
-      <c r="A103" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Transporte</t>
-        </is>
-      </c>
-      <c r="B103" s="216" t="n"/>
-      <c r="C103" s="216" t="n"/>
-      <c r="D103" s="216" t="n"/>
-      <c r="E103" s="216" t="n"/>
-      <c r="F103" s="216" t="n"/>
-      <c r="G103" s="216" t="n"/>
-      <c r="H103" s="216" t="n"/>
+      <c r="A103" s="217" t="n">
+        <v>90</v>
+      </c>
+      <c r="B103" s="218" t="inlineStr">
+        <is>
+          <t>Papeleria &amp; Diseno Grafico</t>
+        </is>
+      </c>
+      <c r="C103" s="218" t="inlineStr">
+        <is>
+          <t>Save the date digital</t>
+        </is>
+      </c>
+      <c r="D103" s="218" t="inlineStr">
+        <is>
+          <t>Folleto digital para anticipar la fecha en redes.</t>
+        </is>
+      </c>
+      <c r="E103" s="219" t="n">
+        <v>1200</v>
+      </c>
+      <c r="F103" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G103" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H103" s="218" t="inlineStr"/>
       <c r="I103" s="216" t="n"/>
     </row>
     <row r="104" ht="18" customHeight="1" s="107">
       <c r="A104" s="217" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B104" s="218" t="inlineStr">
         <is>
-          <t>Transporte</t>
+          <t>Papeleria &amp; Diseno Grafico</t>
         </is>
       </c>
       <c r="C104" s="218" t="inlineStr">
         <is>
-          <t>Transporte de invitados</t>
+          <t>Menús impresos</t>
         </is>
       </c>
       <c r="D104" s="218" t="inlineStr">
         <is>
-          <t>Traslado de invitados en Vans o autobuses ejecutivos.</t>
+          <t>Minutas del menú por persona en cada lugar de mesa.</t>
         </is>
       </c>
       <c r="E104" s="219" t="n">
-        <v>5000</v>
+        <v>800</v>
       </c>
       <c r="F104" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="G104" s="217" t="inlineStr">
@@ -7197,80 +7223,80 @@
       <c r="I104" s="216" t="n"/>
     </row>
     <row r="105" ht="18" customHeight="1" s="107">
-      <c r="A105" s="217" t="n">
-        <v>91</v>
-      </c>
-      <c r="B105" s="218" t="inlineStr">
+      <c r="A105" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Transporte</t>
+        </is>
+      </c>
+      <c r="B105" s="216" t="n"/>
+      <c r="C105" s="216" t="n"/>
+      <c r="D105" s="216" t="n"/>
+      <c r="E105" s="216" t="n"/>
+      <c r="F105" s="216" t="n"/>
+      <c r="G105" s="216" t="n"/>
+      <c r="H105" s="216" t="n"/>
+      <c r="I105" s="216" t="n"/>
+    </row>
+    <row r="106" ht="18" customHeight="1" s="107">
+      <c r="A106" s="217" t="n">
+        <v>92</v>
+      </c>
+      <c r="B106" s="218" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
-      <c r="C105" s="218" t="inlineStr">
-        <is>
-          <t>Auto de lujo / decorado</t>
-        </is>
-      </c>
-      <c r="D105" s="218" t="inlineStr">
-        <is>
-          <t>Auto de gala decorado para el traslado de la novia.</t>
-        </is>
-      </c>
-      <c r="E105" s="219" t="n">
-        <v>3500</v>
-      </c>
-      <c r="F105" s="220" t="inlineStr">
+      <c r="C106" s="218" t="inlineStr">
+        <is>
+          <t>Transporte de invitados</t>
+        </is>
+      </c>
+      <c r="D106" s="218" t="inlineStr">
+        <is>
+          <t>Traslado de invitados en Vans o autobuses ejecutivos.</t>
+        </is>
+      </c>
+      <c r="E106" s="219" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F106" s="220" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="G105" s="217" t="inlineStr">
+      <c r="G106" s="217" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H105" s="218" t="inlineStr"/>
-      <c r="I105" s="216" t="n"/>
-    </row>
-    <row r="106" ht="18" customHeight="1" s="107">
-      <c r="A106" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Staff Operativo</t>
-        </is>
-      </c>
-      <c r="B106" s="216" t="n"/>
-      <c r="C106" s="216" t="n"/>
-      <c r="D106" s="216" t="n"/>
-      <c r="E106" s="216" t="n"/>
-      <c r="F106" s="216" t="n"/>
-      <c r="G106" s="216" t="n"/>
-      <c r="H106" s="216" t="n"/>
+      <c r="H106" s="218" t="inlineStr"/>
       <c r="I106" s="216" t="n"/>
     </row>
     <row r="107" ht="18" customHeight="1" s="107">
       <c r="A107" s="217" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B107" s="218" t="inlineStr">
         <is>
-          <t>Staff Operativo</t>
+          <t>Transporte</t>
         </is>
       </c>
       <c r="C107" s="218" t="inlineStr">
         <is>
-          <t>Banquetes Primavera - Servicio Meseros</t>
+          <t>Auto de lujo / decorado</t>
         </is>
       </c>
       <c r="D107" s="218" t="inlineStr">
         <is>
-          <t>10 meseros uniformados brindando atención personalizada durante 5 horas.</t>
+          <t>Auto de gala decorado para el traslado de la novia.</t>
         </is>
       </c>
       <c r="E107" s="219" t="n">
-        <v>14040</v>
+        <v>3500</v>
       </c>
       <c r="F107" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G107" s="217" t="inlineStr">
@@ -7278,48 +7304,22 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H107" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes")</f>
-        <v/>
-      </c>
+      <c r="H107" s="218" t="inlineStr"/>
       <c r="I107" s="216" t="n"/>
     </row>
     <row r="108" ht="18" customHeight="1" s="107">
-      <c r="A108" s="217" t="n">
-        <v>93</v>
-      </c>
-      <c r="B108" s="218" t="inlineStr">
-        <is>
-          <t>Staff Operativo</t>
-        </is>
-      </c>
-      <c r="C108" s="218" t="inlineStr">
-        <is>
-          <t>Banquetes Primavera - Capitán de Servicio</t>
-        </is>
-      </c>
-      <c r="D108" s="218" t="inlineStr">
-        <is>
-          <t>Capitán coordinador del servicio de alimentos, tiempos de barra y cocina.</t>
-        </is>
-      </c>
-      <c r="E108" s="219" t="n">
-        <v>21060</v>
-      </c>
-      <c r="F108" s="220" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="G108" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H108" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes")</f>
-        <v/>
-      </c>
+      <c r="A108" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Staff Operativo</t>
+        </is>
+      </c>
+      <c r="B108" s="216" t="n"/>
+      <c r="C108" s="216" t="n"/>
+      <c r="D108" s="216" t="n"/>
+      <c r="E108" s="216" t="n"/>
+      <c r="F108" s="216" t="n"/>
+      <c r="G108" s="216" t="n"/>
+      <c r="H108" s="216" t="n"/>
       <c r="I108" s="216" t="n"/>
     </row>
     <row r="109" ht="18" customHeight="1" s="107">
@@ -7333,16 +7333,16 @@
       </c>
       <c r="C109" s="218" t="inlineStr">
         <is>
-          <t>Personal de limpieza</t>
+          <t>Banquetes Primavera - Servicio Meseros</t>
         </is>
       </c>
       <c r="D109" s="218" t="inlineStr">
         <is>
-          <t>Mantenimiento y desinfección de sanitarios durante la gala.</t>
+          <t>10 meseros uniformados brindando atención personalizada durante 5 horas.</t>
         </is>
       </c>
       <c r="E109" s="219" t="n">
-        <v>1500</v>
+        <v>14040</v>
       </c>
       <c r="F109" s="220" t="inlineStr">
         <is>
@@ -7354,49 +7354,75 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H109" s="218" t="inlineStr"/>
+      <c r="H109" s="218">
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes")</f>
+        <v/>
+      </c>
       <c r="I109" s="216" t="n"/>
     </row>
     <row r="110" ht="19.5" customHeight="1" s="107">
-      <c r="A110" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Experiencia &amp; Extras</t>
-        </is>
-      </c>
-      <c r="B110" s="216" t="n"/>
-      <c r="C110" s="216" t="n"/>
-      <c r="D110" s="216" t="n"/>
-      <c r="E110" s="216" t="n"/>
-      <c r="F110" s="216" t="n"/>
-      <c r="G110" s="216" t="n"/>
-      <c r="H110" s="216" t="n"/>
+      <c r="A110" s="217" t="n">
+        <v>95</v>
+      </c>
+      <c r="B110" s="218" t="inlineStr">
+        <is>
+          <t>Staff Operativo</t>
+        </is>
+      </c>
+      <c r="C110" s="218" t="inlineStr">
+        <is>
+          <t>Banquetes Primavera - Capitán de Servicio</t>
+        </is>
+      </c>
+      <c r="D110" s="218" t="inlineStr">
+        <is>
+          <t>Capitán coordinador del servicio de alimentos, tiempos de barra y cocina.</t>
+        </is>
+      </c>
+      <c r="E110" s="219" t="n">
+        <v>21060</v>
+      </c>
+      <c r="F110" s="220" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G110" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H110" s="218">
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes")</f>
+        <v/>
+      </c>
       <c r="I110" s="216" t="n"/>
     </row>
     <row r="111" ht="18" customHeight="1" s="107">
       <c r="A111" s="217" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B111" s="218" t="inlineStr">
         <is>
-          <t>Experiencia &amp; Extras</t>
+          <t>Staff Operativo</t>
         </is>
       </c>
       <c r="C111" s="218" t="inlineStr">
         <is>
-          <t>Recuerdos / Souvenirs</t>
+          <t>Personal de limpieza</t>
         </is>
       </c>
       <c r="D111" s="218" t="inlineStr">
         <is>
-          <t>Detalles temáticos y recuerdos personalizados para invitados.</t>
+          <t>Mantenimiento y desinfección de sanitarios durante la gala.</t>
         </is>
       </c>
       <c r="E111" s="219" t="n">
-        <v>4500</v>
+        <v>1500</v>
       </c>
       <c r="F111" s="220" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="G111" s="217" t="inlineStr">
@@ -7408,38 +7434,18 @@
       <c r="I111" s="216" t="n"/>
     </row>
     <row r="112" ht="18" customHeight="1" s="107">
-      <c r="A112" s="217" t="n">
-        <v>96</v>
-      </c>
-      <c r="B112" s="218" t="inlineStr">
-        <is>
-          <t>Experiencia &amp; Extras</t>
-        </is>
-      </c>
-      <c r="C112" s="218" t="inlineStr">
-        <is>
-          <t>Show pirotécnico frío</t>
-        </is>
-      </c>
-      <c r="D112" s="218" t="inlineStr">
-        <is>
-          <t>Chispas de luz fría de interior para el baile y vals.</t>
-        </is>
-      </c>
-      <c r="E112" s="219" t="n">
-        <v>3000</v>
-      </c>
-      <c r="F112" s="220" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="G112" s="217" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H112" s="218" t="inlineStr"/>
+      <c r="A112" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Experiencia &amp; Extras</t>
+        </is>
+      </c>
+      <c r="B112" s="216" t="n"/>
+      <c r="C112" s="216" t="n"/>
+      <c r="D112" s="216" t="n"/>
+      <c r="E112" s="216" t="n"/>
+      <c r="F112" s="216" t="n"/>
+      <c r="G112" s="216" t="n"/>
+      <c r="H112" s="216" t="n"/>
       <c r="I112" s="216" t="n"/>
     </row>
     <row r="113" ht="18" customHeight="1" s="107">
@@ -7453,16 +7459,16 @@
       </c>
       <c r="C113" s="218" t="inlineStr">
         <is>
-          <t>Letras gigantes LED</t>
+          <t>Recuerdos / Souvenirs</t>
         </is>
       </c>
       <c r="D113" s="218" t="inlineStr">
         <is>
-          <t>Renta de letras gigantes iluminadas con iniciales (pista).</t>
+          <t>Detalles temáticos y recuerdos personalizados para invitados.</t>
         </is>
       </c>
       <c r="E113" s="219" t="n">
-        <v>2500</v>
+        <v>4500</v>
       </c>
       <c r="F113" s="220" t="inlineStr">
         <is>
@@ -7478,45 +7484,65 @@
       <c r="I113" s="216" t="n"/>
     </row>
     <row r="114" ht="18" customHeight="1" s="107">
-      <c r="A114" s="215" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Servicios Administrativos</t>
-        </is>
-      </c>
-      <c r="B114" s="216" t="n"/>
-      <c r="C114" s="216" t="n"/>
-      <c r="D114" s="216" t="n"/>
-      <c r="E114" s="216" t="n"/>
-      <c r="F114" s="216" t="n"/>
-      <c r="G114" s="216" t="n"/>
-      <c r="H114" s="216" t="n"/>
+      <c r="A114" s="217" t="n">
+        <v>98</v>
+      </c>
+      <c r="B114" s="218" t="inlineStr">
+        <is>
+          <t>Experiencia &amp; Extras</t>
+        </is>
+      </c>
+      <c r="C114" s="218" t="inlineStr">
+        <is>
+          <t>Show pirotécnico frío</t>
+        </is>
+      </c>
+      <c r="D114" s="218" t="inlineStr">
+        <is>
+          <t>Chispas de luz fría de interior para el baile y vals.</t>
+        </is>
+      </c>
+      <c r="E114" s="219" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F114" s="220" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="G114" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H114" s="218" t="inlineStr"/>
       <c r="I114" s="216" t="n"/>
     </row>
     <row r="115" ht="15" customHeight="1" s="107">
       <c r="A115" s="217" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B115" s="218" t="inlineStr">
         <is>
-          <t>Servicios Administrativos</t>
+          <t>Experiencia &amp; Extras</t>
         </is>
       </c>
       <c r="C115" s="218" t="inlineStr">
         <is>
-          <t>Seguro del evento</t>
+          <t>Letras gigantes LED</t>
         </is>
       </c>
       <c r="D115" s="218" t="inlineStr">
         <is>
-          <t>Póliza contra cancelación, accidentes o imprevistos de clima.</t>
+          <t>Renta de letras gigantes iluminadas con iniciales (pista).</t>
         </is>
       </c>
       <c r="E115" s="219" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="F115" s="220" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="G115" s="217" t="inlineStr">
@@ -7528,60 +7554,110 @@
       <c r="I115" s="216" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="217" t="n">
-        <v>99</v>
-      </c>
-      <c r="B116" s="218" t="inlineStr">
+      <c r="A116" s="215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Servicios Administrativos</t>
+        </is>
+      </c>
+      <c r="B116" s="216" t="n"/>
+      <c r="C116" s="216" t="n"/>
+      <c r="D116" s="216" t="n"/>
+      <c r="E116" s="216" t="n"/>
+      <c r="F116" s="216" t="n"/>
+      <c r="G116" s="216" t="n"/>
+      <c r="H116" s="216" t="n"/>
+      <c r="I116" s="216" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="217" t="n">
+        <v>100</v>
+      </c>
+      <c r="B117" s="218" t="inlineStr">
         <is>
           <t>Servicios Administrativos</t>
         </is>
       </c>
-      <c r="C116" s="218" t="inlineStr">
+      <c r="C117" s="218" t="inlineStr">
+        <is>
+          <t>Seguro del evento</t>
+        </is>
+      </c>
+      <c r="D117" s="218" t="inlineStr">
+        <is>
+          <t>Póliza contra cancelación, accidentes o imprevistos de clima.</t>
+        </is>
+      </c>
+      <c r="E117" s="219" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F117" s="220" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="G117" s="217" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H117" s="218" t="inlineStr"/>
+      <c r="I117" s="216" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="217" t="n">
+        <v>101</v>
+      </c>
+      <c r="B118" s="218" t="inlineStr">
+        <is>
+          <t>Servicios Administrativos</t>
+        </is>
+      </c>
+      <c r="C118" s="218" t="inlineStr">
         <is>
           <t>Contratos y gestión legal</t>
         </is>
       </c>
-      <c r="D116" s="218" t="inlineStr">
+      <c r="D118" s="218" t="inlineStr">
         <is>
           <t>Control de contratos de expositores y logística legal.</t>
         </is>
       </c>
-      <c r="E116" s="219" t="n">
+      <c r="E118" s="219" t="n">
         <v>1500</v>
       </c>
-      <c r="F116" s="220" t="inlineStr">
+      <c r="F118" s="220" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="G116" s="217" t="inlineStr">
+      <c r="G118" s="217" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H116" s="218" t="inlineStr"/>
-      <c r="I116" s="216" t="n"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="221" t="inlineStr">
-        <is>
-          <t>TOTAL SERVICIOS SELECCIONADOS (99 servicios disponibles)</t>
-        </is>
-      </c>
-      <c r="B117" s="216" t="n"/>
-      <c r="C117" s="216" t="n"/>
-      <c r="D117" s="216" t="n"/>
-      <c r="E117" s="222">
-        <f>SUMIF(G4:G116,"✓",E4:E116)</f>
-        <v/>
-      </c>
-      <c r="F117" s="223">
-        <f>COUNTIF(G4:G116,"✓") &amp; " seleccionados"</f>
-        <v/>
-      </c>
-      <c r="G117" s="216" t="n"/>
-      <c r="H117" s="216" t="n"/>
-      <c r="I117" s="216" t="n"/>
+      <c r="H118" s="218" t="inlineStr"/>
+      <c r="I118" s="216" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="216" t="inlineStr">
+        <is>
+          <t>TOTAL SERVICIOS SELECCIONADOS (101 servicios disponibles)</t>
+        </is>
+      </c>
+      <c r="B119" s="216" t="n"/>
+      <c r="C119" s="216" t="n"/>
+      <c r="D119" s="216" t="n"/>
+      <c r="E119" s="216">
+        <f>SUMIF(G4:G118,"✓",E4:E118)</f>
+        <v/>
+      </c>
+      <c r="F119" s="216">
+        <f>COUNTIF(G4:G118,"✓") &amp; " seleccionados"</f>
+        <v/>
+      </c>
+      <c r="G119" s="216" t="n"/>
+      <c r="H119" s="216" t="n"/>
+      <c r="I119" s="216" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -13405,7 +13481,7 @@
         </is>
       </c>
       <c r="C8" s="210">
-        <f>'📦 Catálogo'!E117</f>
+        <f>'📦 Catálogo'!E119</f>
         <v/>
       </c>
       <c r="D8" s="114" t="n"/>

</xml_diff>

<commit_message>
fix: corregir todos los enlaces de banquetes y paquetes en el excel usando urls reales del sitemap
</commit_message>
<xml_diff>
--- a/assets/Smart_Event_Planner_Pro.xlsx
+++ b/assets/Smart_Event_Planner_Pro.xlsx
@@ -3770,7 +3770,7 @@
         </is>
       </c>
       <c r="H5" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Centro Presidente")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Locaciones")</f>
         <v/>
       </c>
       <c r="I5" s="216" t="n"/>
@@ -3808,7 +3808,7 @@
         </is>
       </c>
       <c r="H6" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Salón Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Locaciones")</f>
         <v/>
       </c>
       <c r="I6" s="216" t="n"/>
@@ -3846,7 +3846,7 @@
         </is>
       </c>
       <c r="H7" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Salón Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Locaciones")</f>
         <v/>
       </c>
       <c r="I7" s="216" t="n"/>
@@ -3884,7 +3884,7 @@
         </is>
       </c>
       <c r="H8" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Salón Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Locaciones")</f>
         <v/>
       </c>
       <c r="I8" s="216" t="n"/>
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="H9" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Salón Calesa")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Locaciones")</f>
         <v/>
       </c>
       <c r="I9" s="216" t="n"/>
@@ -3960,7 +3960,7 @@
         </is>
       </c>
       <c r="H10" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Salón Calesa")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/venues/","Ver Locaciones")</f>
         <v/>
       </c>
       <c r="I10" s="216" t="n"/>
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="H18" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Combos Oficiales")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/","Ver Paquetes")</f>
         <v/>
       </c>
       <c r="I18" s="216" t="n"/>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="H19" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Combos Oficiales")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/","Ver Paquetes")</f>
         <v/>
       </c>
       <c r="I19" s="216" t="n"/>
@@ -4299,7 +4299,7 @@
         </is>
       </c>
       <c r="H20" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Menus")</f>
         <v/>
       </c>
       <c r="I20" s="216" t="n"/>
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="H21" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Menus")</f>
         <v/>
       </c>
       <c r="I21" s="216" t="n"/>
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="H22" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes Primavera")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Menus")</f>
         <v/>
       </c>
       <c r="I22" s="216" t="n"/>
@@ -5998,7 +5998,7 @@
       </c>
       <c r="D68" s="218" t="inlineStr">
         <is>
-          <t>Corte y arreglo de barba profesional para el novio el gran día.</t>
+          <t>Corte y arreglo de barra profesional para el novio el gran día.</t>
         </is>
       </c>
       <c r="E68" s="219" t="n">
@@ -6451,7 +6451,7 @@
         </is>
       </c>
       <c r="H82" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Jessy &amp; Richard")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Servicios")</f>
         <v/>
       </c>
       <c r="I82" s="216" t="n"/>
@@ -6489,7 +6489,7 @@
         </is>
       </c>
       <c r="H83" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Jessy &amp; Richard")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/wedding-event-planning/","Ver Servicios")</f>
         <v/>
       </c>
       <c r="I83" s="216" t="n"/>
@@ -7355,7 +7355,7 @@
         </is>
       </c>
       <c r="H109" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Menus")</f>
         <v/>
       </c>
       <c r="I109" s="216" t="n"/>
@@ -7393,7 +7393,7 @@
         </is>
       </c>
       <c r="H110" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Banquetes")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/banquetes-primavera/","Ver Menus")</f>
         <v/>
       </c>
       <c r="I110" s="216" t="n"/>

</xml_diff>

<commit_message>
fix: corregir el enlace de paquetes a la url paquetes-primavera compartida por el usuario
</commit_message>
<xml_diff>
--- a/assets/Smart_Event_Planner_Pro.xlsx
+++ b/assets/Smart_Event_Planner_Pro.xlsx
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="H18" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/","Ver Paquetes")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/paquetes-primavera/","Ver Paquetes")</f>
         <v/>
       </c>
       <c r="I18" s="216" t="n"/>
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="H19" s="218">
-        <f>HYPERLINK("https://primaveraeventsgroup.com/987509796-2/","Ver Paquetes")</f>
+        <f>HYPERLINK("https://primaveraeventsgroup.com/paquetes-primavera/","Ver Paquetes")</f>
         <v/>
       </c>
       <c r="I19" s="216" t="n"/>
@@ -6700,7 +6700,7 @@
       </c>
       <c r="D89" s="218" t="inlineStr">
         <is>
-          <t>Panel circular con set de globos y luces de neón decorativas.</t>
+          <t>Panel circular con set de globos and luces de neón decorativas.</t>
         </is>
       </c>
       <c r="E89" s="219" t="n">

</xml_diff>